<commit_message>
Work on second rally
</commit_message>
<xml_diff>
--- a/Rallies.xlsx
+++ b/Rallies.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="67">
   <si>
     <t>Year</t>
   </si>
@@ -178,13 +178,43 @@
     <t>0, 6</t>
   </si>
   <si>
-    <t>Date</t>
-  </si>
-  <si>
     <t>19-21 August</t>
   </si>
   <si>
     <t>Morning, Afternoon</t>
+  </si>
+  <si>
+    <t>22-26 February</t>
+  </si>
+  <si>
+    <t>// 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>// 5</t>
+  </si>
+  <si>
+    <t>// 6</t>
+  </si>
+  <si>
+    <t>Fog, Afternoon, Sunset</t>
+  </si>
+  <si>
+    <t>2, 6, 0</t>
+  </si>
+  <si>
+    <t>Has pilot picture</t>
+  </si>
+  <si>
+    <t>Has car picture</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Date (for weather)</t>
   </si>
 </sst>
 </file>
@@ -229,7 +259,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -239,12 +269,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -277,26 +301,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -333,21 +348,35 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="51">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -388,6 +417,312 @@
       <fill>
         <patternFill>
           <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor auto="1"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor auto="1"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor auto="1"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor auto="1"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor auto="1"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -688,446 +1023,492 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:T25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="7" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9" style="5" customWidth="1"/>
+    <col min="3" max="3" width="9" style="3" customWidth="1"/>
     <col min="4" max="4" width="15.81640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.90625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.81640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="17.7265625" style="1" customWidth="1"/>
     <col min="7" max="7" width="12.1796875" style="1" customWidth="1"/>
     <col min="8" max="8" width="14.54296875" style="1" customWidth="1"/>
     <col min="9" max="9" width="7.1796875" style="1" customWidth="1"/>
     <col min="10" max="10" width="12.26953125" style="1" customWidth="1"/>
     <col min="11" max="11" width="9.81640625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="18.7265625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="16.7265625" style="1" customWidth="1"/>
     <col min="13" max="13" width="62" style="1" customWidth="1"/>
-    <col min="14" max="14" width="7.81640625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="9.08984375" style="1" customWidth="1"/>
+    <col min="14" max="15" width="8.453125" style="1" customWidth="1"/>
     <col min="16" max="16" width="9.1796875" style="1" customWidth="1"/>
     <col min="17" max="18" width="13.90625" style="1" customWidth="1"/>
-    <col min="19" max="16384" width="8.7265625" style="1"/>
+    <col min="19" max="19" width="13.453125" style="1" customWidth="1"/>
+    <col min="20" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="4" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:20" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="R1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="S1" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="78" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="16">
+        <v>1966</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F2" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="16">
+        <v>1966</v>
+      </c>
+      <c r="H2" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="I2" s="16">
+        <v>0</v>
+      </c>
+      <c r="J2" s="16">
         <v>2</v>
       </c>
-      <c r="G1" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="M1" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="O1" s="9" t="s">
+      <c r="K2" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L2" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="M2" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="O2" s="16"/>
+      <c r="P2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" ht="74.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="B3" s="16">
+        <v>1967</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="16">
+        <v>1967</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="I3" s="16">
+        <v>1</v>
+      </c>
+      <c r="J3" s="16">
+        <v>0</v>
+      </c>
+      <c r="K3" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L3" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" ht="81.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="16">
+        <v>1968</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="16">
+        <v>1969</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="I4" s="16">
+        <v>5</v>
+      </c>
+      <c r="J4" s="16">
+        <v>4</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L4" s="17"/>
+      <c r="M4" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" ht="91" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="16">
+        <v>1970</v>
+      </c>
+      <c r="C5" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="R1" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" ht="78" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="2">
+      <c r="D5" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="16">
         <v>1966</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="21">
-        <v>1966</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I2" s="2">
-        <v>0</v>
-      </c>
-      <c r="J2" s="2">
+      <c r="H5" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" s="16">
+        <v>1</v>
+      </c>
+      <c r="J5" s="16">
         <v>2</v>
       </c>
-      <c r="K2" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="O2" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="P2" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" ht="74.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="2">
-        <v>1967</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="21">
-        <v>1967</v>
-      </c>
-      <c r="H3" s="6" t="s">
+      <c r="K5" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L5" s="17"/>
+      <c r="M5" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="S5" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K6" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="R6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="S6" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="Q7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="R7" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="S7" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="I3" s="2">
-        <v>1</v>
-      </c>
-      <c r="J3" s="21">
-        <v>0</v>
-      </c>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="O3" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="P3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q3" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" ht="81.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2">
-        <v>1968</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="21">
-        <v>1969</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="I4" s="21">
-        <v>5</v>
-      </c>
-      <c r="J4" s="21">
-        <v>4</v>
-      </c>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="O4" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="P4" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q4" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="R4" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" ht="91" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2">
-        <v>1970</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="21">
-        <v>1966</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="I5" s="21">
-        <v>1</v>
-      </c>
-      <c r="J5" s="21">
-        <v>2</v>
-      </c>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="O5" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="P5" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="Q5" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="R5" s="5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="O6" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="P6" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q6" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="R6" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12"/>
-      <c r="P7" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q7" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="R7" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="P8" s="9" t="s">
+    </row>
+    <row r="8" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="Q8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="R8" s="5" t="s">
+      <c r="S8" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-      <c r="P9" s="11"/>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="18"/>
-      <c r="P10" s="5"/>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
-      <c r="P11" s="5"/>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="L12" s="5"/>
-      <c r="P12" s="5"/>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="F13" s="5"/>
-      <c r="P13" s="5"/>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="P9" s="8"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="15"/>
+      <c r="P10" s="3"/>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="P11" s="3"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="L12" s="3"/>
+      <c r="P12" s="3"/>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="F13" s="3"/>
+      <c r="P13" s="3"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="14"/>
-      <c r="M18" s="4"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11"/>
+      <c r="M18" s="2"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A19" s="16"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="16"/>
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="13"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="O24" s="9"/>
+      <c r="O24" s="6"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="O25" s="9"/>
-      <c r="P25" s="8"/>
+      <c r="O25" s="6"/>
+      <c r="P25" s="5"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:O5">
+    <cfRule type="containsBlanks" dxfId="9" priority="2">
+      <formula>LEN(TRIM(A2))=0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="1">
+      <formula>COUNTA($A2:$O2)=COLUMNS($A2:$O2)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P8 C2:C5 G19 H7:H8 G9">
-      <formula1>$P$1:$P$8</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q8 G9 H7:H8 G19 C2:C5">
+      <formula1>$Q$1:$Q$8</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H5">
-      <formula1>$R$2:$R$8</formula1>
+      <formula1>$S$2:$S$8</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A19 A2:A5 A7:A9">
-      <formula1>$O$1:$O$6</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A19 A7:A9 A2:A5">
+      <formula1>$P$1:$P$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="K3" twoDigitTextYear="1"/>
+  </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="21" operator="containsText" id="{DA6F5A75-15ED-44BA-BB89-65868BD70EF4}">
-            <xm:f>NOT(ISERROR(SEARCH($O$6,A7)))</xm:f>
-            <xm:f>$O$6</xm:f>
+          <x14:cfRule type="containsText" priority="30" operator="containsText" id="{DA6F5A75-15ED-44BA-BB89-65868BD70EF4}">
+            <xm:f>NOT(ISERROR(SEARCH($P$6,A7)))</xm:f>
+            <xm:f>$P$6</xm:f>
             <x14:dxf>
               <fill>
                 <patternFill>
@@ -1136,9 +1517,9 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="22" operator="containsText" id="{E2646601-D923-4D79-BA19-07772457BD39}">
-            <xm:f>NOT(ISERROR(SEARCH($O$5,A7)))</xm:f>
-            <xm:f>$O$5</xm:f>
+          <x14:cfRule type="containsText" priority="31" operator="containsText" id="{E2646601-D923-4D79-BA19-07772457BD39}">
+            <xm:f>NOT(ISERROR(SEARCH($P$5,A7)))</xm:f>
+            <xm:f>$P$5</xm:f>
             <x14:dxf>
               <fill>
                 <patternFill>
@@ -1147,9 +1528,9 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="23" operator="containsText" id="{7CBFFB87-A85C-408E-AEE4-4F09CD3A5E7D}">
-            <xm:f>NOT(ISERROR(SEARCH($O$4,A7)))</xm:f>
-            <xm:f>$O$4</xm:f>
+          <x14:cfRule type="containsText" priority="32" operator="containsText" id="{7CBFFB87-A85C-408E-AEE4-4F09CD3A5E7D}">
+            <xm:f>NOT(ISERROR(SEARCH($P$4,A7)))</xm:f>
+            <xm:f>$P$4</xm:f>
             <x14:dxf>
               <fill>
                 <patternFill>
@@ -1158,9 +1539,9 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="24" operator="containsText" id="{CBA09518-7F8B-43A7-A676-37830780E4DD}">
-            <xm:f>NOT(ISERROR(SEARCH($O$3,A7)))</xm:f>
-            <xm:f>$O$3</xm:f>
+          <x14:cfRule type="containsText" priority="33" operator="containsText" id="{CBA09518-7F8B-43A7-A676-37830780E4DD}">
+            <xm:f>NOT(ISERROR(SEARCH($P$3,A7)))</xm:f>
+            <xm:f>$P$3</xm:f>
             <x14:dxf>
               <fill>
                 <patternFill>
@@ -1169,9 +1550,9 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="25" operator="containsText" id="{4BDEC88A-D0B4-4531-8A76-36189880D171}">
-            <xm:f>NOT(ISERROR(SEARCH($O$2,A7)))</xm:f>
-            <xm:f>$O$2</xm:f>
+          <x14:cfRule type="containsText" priority="34" operator="containsText" id="{4BDEC88A-D0B4-4531-8A76-36189880D171}">
+            <xm:f>NOT(ISERROR(SEARCH($P$2,A7)))</xm:f>
+            <xm:f>$P$2</xm:f>
             <x14:dxf>
               <fill>
                 <patternFill>
@@ -1180,9 +1561,9 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="containsText" priority="26" operator="containsText" id="{DAF95EAF-2CFF-4893-A297-20F654754CD1}">
-            <xm:f>NOT(ISERROR(SEARCH($O$1,A7)))</xm:f>
-            <xm:f>$O$1</xm:f>
+          <x14:cfRule type="containsText" priority="35" operator="containsText" id="{DAF95EAF-2CFF-4893-A297-20F654754CD1}">
+            <xm:f>NOT(ISERROR(SEARCH($P$1,A7)))</xm:f>
+            <xm:f>$P$1</xm:f>
             <x14:dxf>
               <fill>
                 <patternFill>

</xml_diff>

<commit_message>
Add rally 3 group 2
</commit_message>
<xml_diff>
--- a/Rallies.xlsx
+++ b/Rallies.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="73">
   <si>
     <t>Year</t>
   </si>
@@ -215,6 +215,24 @@
   </si>
   <si>
     <t>Date (for weather)</t>
+  </si>
+  <si>
+    <t>2-5 May</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Italy</t>
+  </si>
+  <si>
+    <t>West Germany</t>
+  </si>
+  <si>
+    <t>Rain, Sunset, Fog, Afternoon</t>
+  </si>
+  <si>
+    <t>0, 5, 3, 11</t>
   </si>
 </sst>
 </file>
@@ -354,14 +372,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFFF00"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -662,31 +680,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T58"/>
+  <dimension ref="A1:U58"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="7" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9" style="4" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="14.81640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17.7265625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1796875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.54296875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="7.1796875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="12.26953125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.81640625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16.7265625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="62" style="1" customWidth="1"/>
-    <col min="14" max="15" width="8.453125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="9.1796875" style="1" customWidth="1"/>
-    <col min="17" max="18" width="13.90625" style="1" customWidth="1"/>
-    <col min="19" max="19" width="13.453125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="14.6328125" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="8.7265625" style="1"/>
+    <col min="3" max="4" width="9" style="4" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14.81640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.7265625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="14.54296875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.1796875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12.26953125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.81640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="16.7265625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="62" style="1" customWidth="1"/>
+    <col min="15" max="16" width="8.453125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="9.1796875" style="1" customWidth="1"/>
+    <col min="18" max="19" width="13.90625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="13.453125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="14.6328125" style="1" customWidth="1"/>
+    <col min="22" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="3" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" s="3" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>33</v>
       </c>
@@ -697,58 +715,61 @@
         <v>34</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="Q1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="R1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="T1" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="78" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" ht="78" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
         <v>12</v>
       </c>
@@ -759,55 +780,58 @@
         <v>3</v>
       </c>
       <c r="D2" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="F2" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="G2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="10">
+      <c r="H2" s="10">
         <v>1966</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="I2" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="I2" s="10">
+      <c r="J2" s="10">
         <v>0</v>
       </c>
-      <c r="J2" s="10">
+      <c r="K2" s="10">
         <v>2</v>
       </c>
-      <c r="K2" s="10" t="s">
+      <c r="L2" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="M2" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="M2" s="11" t="s">
+      <c r="N2" s="11" t="s">
         <v>31</v>
-      </c>
-      <c r="N2" s="10" t="s">
-        <v>65</v>
       </c>
       <c r="O2" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="P2" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="R2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="S2" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="74.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" ht="74.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>12</v>
       </c>
@@ -818,55 +842,58 @@
         <v>13</v>
       </c>
       <c r="D3" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="10">
+      <c r="H3" s="10">
         <v>1967</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="I3" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="I3" s="10">
+      <c r="J3" s="10">
         <v>1</v>
       </c>
-      <c r="J3" s="10">
+      <c r="K3" s="10">
         <v>0</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="L3" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="L3" s="11" t="s">
+      <c r="M3" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="M3" s="11" t="s">
+      <c r="N3" s="11" t="s">
         <v>32</v>
-      </c>
-      <c r="N3" s="10" t="s">
-        <v>65</v>
       </c>
       <c r="O3" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P3" s="7" t="s">
+      <c r="P3" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="7" t="s">
+      <c r="R3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="R3" s="6" t="s">
+      <c r="S3" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="S3" s="4" t="s">
+      <c r="T3" s="4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="81.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" ht="81.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
         <v>12</v>
       </c>
@@ -877,47 +904,58 @@
         <v>8</v>
       </c>
       <c r="D4" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="10"/>
       <c r="F4" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="10">
+      <c r="H4" s="10">
         <v>1969</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="I4" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I4" s="10">
+      <c r="J4" s="10">
         <v>5</v>
       </c>
-      <c r="J4" s="10">
-        <v>4</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="L4" s="11"/>
+      <c r="K4" s="10">
+        <v>0</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>72</v>
+      </c>
       <c r="M4" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="N4" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="7" t="s">
+      <c r="O4" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q4" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="Q4" s="7" t="s">
+      <c r="R4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="R4" s="6" t="s">
+      <c r="S4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="S4" s="4" t="s">
+      <c r="T4" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="91" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" ht="91" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
         <v>12</v>
       </c>
@@ -928,1224 +966,1280 @@
         <v>3</v>
       </c>
       <c r="D5" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="10"/>
+      <c r="G5" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="10">
+      <c r="H5" s="10">
         <v>1966</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="I5" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="I5" s="10">
+      <c r="J5" s="10">
         <v>1</v>
       </c>
-      <c r="J5" s="10">
+      <c r="K5" s="10">
         <v>2</v>
       </c>
-      <c r="K5" s="10" t="s">
+      <c r="L5" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11" t="s">
+      <c r="M5" s="11"/>
+      <c r="N5" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="N5" s="10"/>
       <c r="O5" s="10"/>
-      <c r="P5" s="7" t="s">
+      <c r="P5" s="10"/>
+      <c r="Q5" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="R5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="R5" s="6" t="s">
+      <c r="S5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="S5" s="4" t="s">
+      <c r="T5" s="4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
-      <c r="E6" s="10"/>
+      <c r="E6" s="11"/>
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="11"/>
       <c r="J6" s="10"/>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="10"/>
+      <c r="L6" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="L6" s="11"/>
       <c r="M6" s="11"/>
-      <c r="N6" s="10"/>
+      <c r="N6" s="11"/>
       <c r="O6" s="10"/>
-      <c r="P6" s="7" t="s">
+      <c r="P6" s="10"/>
+      <c r="Q6" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="Q6" s="7" t="s">
+      <c r="R6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="R6" s="6" t="s">
+      <c r="S6" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="S6" s="4" t="s">
+      <c r="T6" s="4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="11"/>
       <c r="D7" s="11"/>
-      <c r="E7" s="10"/>
+      <c r="E7" s="11"/>
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="11"/>
       <c r="J7" s="10"/>
-      <c r="K7" s="2" t="s">
+      <c r="K7" s="10"/>
+      <c r="L7" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="L7" s="11"/>
       <c r="M7" s="11"/>
-      <c r="N7" s="10"/>
+      <c r="N7" s="11"/>
       <c r="O7" s="10"/>
-      <c r="Q7" s="7" t="s">
+      <c r="P7" s="10"/>
+      <c r="R7" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="R7" s="6" t="s">
+      <c r="S7" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="S7" s="4" t="s">
+      <c r="T7" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
         <v>12</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
-      <c r="E8" s="10"/>
+      <c r="E8" s="11"/>
       <c r="F8" s="10"/>
       <c r="G8" s="10"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="11"/>
       <c r="J8" s="10"/>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="10"/>
+      <c r="L8" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="L8" s="11"/>
       <c r="M8" s="11"/>
-      <c r="N8" s="10"/>
+      <c r="N8" s="11"/>
       <c r="O8" s="10"/>
-      <c r="Q8" s="7" t="s">
+      <c r="P8" s="10"/>
+      <c r="R8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="S8" s="4" t="s">
+      <c r="T8" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
-      <c r="E9" s="10"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="10"/>
       <c r="G9" s="10"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="11"/>
       <c r="J9" s="10"/>
-      <c r="K9" s="2" t="s">
+      <c r="K9" s="10"/>
+      <c r="L9" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="L9" s="11"/>
       <c r="M9" s="11"/>
-      <c r="N9" s="10"/>
+      <c r="N9" s="11"/>
       <c r="O9" s="10"/>
-      <c r="P9" s="9"/>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="P9" s="10"/>
+      <c r="Q9" s="9"/>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
-      <c r="E10" s="10"/>
+      <c r="E10" s="11"/>
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="11"/>
       <c r="J10" s="10"/>
-      <c r="K10" s="13">
+      <c r="K10" s="10"/>
+      <c r="L10" s="13">
         <v>3</v>
       </c>
-      <c r="L10" s="11"/>
       <c r="M10" s="11"/>
-      <c r="N10" s="10"/>
+      <c r="N10" s="11"/>
       <c r="O10" s="10"/>
-      <c r="P10" s="4"/>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="P10" s="10"/>
+      <c r="Q10" s="4"/>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
-      <c r="E11" s="10"/>
+      <c r="E11" s="11"/>
       <c r="F11" s="10"/>
       <c r="G11" s="10"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="11"/>
       <c r="J11" s="10"/>
-      <c r="K11" s="13">
+      <c r="K11" s="10"/>
+      <c r="L11" s="13">
         <v>3</v>
       </c>
-      <c r="L11" s="11"/>
       <c r="M11" s="11"/>
-      <c r="N11" s="10"/>
+      <c r="N11" s="11"/>
       <c r="O11" s="10"/>
-      <c r="P11" s="4"/>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="P11" s="10"/>
+      <c r="Q11" s="4"/>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="11"/>
       <c r="D12" s="11"/>
-      <c r="E12" s="10"/>
+      <c r="E12" s="11"/>
       <c r="F12" s="10"/>
       <c r="G12" s="10"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="11"/>
       <c r="J12" s="10"/>
-      <c r="K12" s="13">
+      <c r="K12" s="10"/>
+      <c r="L12" s="13">
         <v>4</v>
       </c>
-      <c r="L12" s="11"/>
       <c r="M12" s="11"/>
-      <c r="N12" s="10"/>
+      <c r="N12" s="11"/>
       <c r="O12" s="10"/>
-      <c r="P12" s="4"/>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="P12" s="10"/>
+      <c r="Q12" s="4"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
-      <c r="E13" s="10"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="11"/>
       <c r="J13" s="10"/>
-      <c r="K13" s="13">
+      <c r="K13" s="10"/>
+      <c r="L13" s="13">
         <v>4</v>
       </c>
-      <c r="L13" s="11"/>
       <c r="M13" s="11"/>
-      <c r="N13" s="10"/>
+      <c r="N13" s="11"/>
       <c r="O13" s="10"/>
-      <c r="P13" s="4"/>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="P13" s="10"/>
+      <c r="Q13" s="4"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
-      <c r="E14" s="10"/>
+      <c r="E14" s="11"/>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="11"/>
       <c r="J14" s="10"/>
-      <c r="K14" s="13">
+      <c r="K14" s="10"/>
+      <c r="L14" s="13">
         <v>4</v>
       </c>
-      <c r="L14" s="11"/>
       <c r="M14" s="11"/>
-      <c r="N14" s="10"/>
+      <c r="N14" s="11"/>
       <c r="O14" s="10"/>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="P14" s="10"/>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11"/>
-      <c r="E15" s="10"/>
+      <c r="E15" s="11"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="11"/>
       <c r="J15" s="10"/>
-      <c r="K15" s="13">
+      <c r="K15" s="10"/>
+      <c r="L15" s="13">
         <v>5</v>
       </c>
-      <c r="L15" s="11"/>
       <c r="M15" s="11"/>
-      <c r="N15" s="10"/>
+      <c r="N15" s="11"/>
       <c r="O15" s="10"/>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="P15" s="10"/>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
-      <c r="E16" s="10"/>
+      <c r="E16" s="11"/>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="11"/>
       <c r="J16" s="10"/>
-      <c r="K16" s="13">
+      <c r="K16" s="10"/>
+      <c r="L16" s="13">
         <v>5</v>
       </c>
-      <c r="L16" s="11"/>
       <c r="M16" s="11"/>
-      <c r="N16" s="10"/>
+      <c r="N16" s="11"/>
       <c r="O16" s="10"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P16" s="10"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="10"/>
       <c r="C17" s="11"/>
       <c r="D17" s="11"/>
-      <c r="E17" s="10"/>
+      <c r="E17" s="11"/>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="11"/>
       <c r="J17" s="10"/>
-      <c r="K17" s="13">
+      <c r="K17" s="10"/>
+      <c r="L17" s="13">
         <v>6</v>
       </c>
-      <c r="L17" s="11"/>
       <c r="M17" s="11"/>
-      <c r="N17" s="10"/>
+      <c r="N17" s="11"/>
       <c r="O17" s="10"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P17" s="10"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="11"/>
       <c r="D18" s="11"/>
-      <c r="E18" s="10"/>
+      <c r="E18" s="11"/>
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="11"/>
       <c r="J18" s="10"/>
-      <c r="K18" s="14">
+      <c r="K18" s="10"/>
+      <c r="L18" s="14">
         <v>6</v>
       </c>
-      <c r="L18" s="11"/>
       <c r="M18" s="11"/>
-      <c r="N18" s="10"/>
+      <c r="N18" s="11"/>
       <c r="O18" s="10"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P18" s="10"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="10"/>
       <c r="C19" s="11"/>
       <c r="D19" s="11"/>
-      <c r="E19" s="10"/>
+      <c r="E19" s="11"/>
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="11"/>
       <c r="J19" s="10"/>
-      <c r="K19" s="15">
+      <c r="K19" s="10"/>
+      <c r="L19" s="15">
         <v>3</v>
       </c>
-      <c r="L19" s="11"/>
       <c r="M19" s="11"/>
-      <c r="N19" s="10"/>
+      <c r="N19" s="11"/>
       <c r="O19" s="10"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P19" s="10"/>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A20" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B20" s="10"/>
       <c r="C20" s="11"/>
       <c r="D20" s="11"/>
-      <c r="E20" s="10"/>
+      <c r="E20" s="11"/>
       <c r="F20" s="10"/>
       <c r="G20" s="10"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="11"/>
       <c r="J20" s="10"/>
-      <c r="K20" s="13">
+      <c r="K20" s="10"/>
+      <c r="L20" s="13">
         <v>4</v>
       </c>
-      <c r="L20" s="11"/>
       <c r="M20" s="11"/>
-      <c r="N20" s="10"/>
+      <c r="N20" s="11"/>
       <c r="O20" s="10"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P20" s="10"/>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B21" s="10"/>
       <c r="C21" s="11"/>
       <c r="D21" s="11"/>
-      <c r="E21" s="10"/>
+      <c r="E21" s="11"/>
       <c r="F21" s="10"/>
       <c r="G21" s="10"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="11"/>
       <c r="J21" s="10"/>
-      <c r="K21" s="13">
+      <c r="K21" s="10"/>
+      <c r="L21" s="13">
         <v>4</v>
       </c>
-      <c r="L21" s="11"/>
       <c r="M21" s="11"/>
-      <c r="N21" s="10"/>
+      <c r="N21" s="11"/>
       <c r="O21" s="10"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P21" s="10"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="11"/>
       <c r="D22" s="11"/>
-      <c r="E22" s="10"/>
+      <c r="E22" s="11"/>
       <c r="F22" s="10"/>
       <c r="G22" s="10"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="11"/>
       <c r="J22" s="10"/>
-      <c r="K22" s="13">
+      <c r="K22" s="10"/>
+      <c r="L22" s="13">
         <v>4</v>
       </c>
-      <c r="L22" s="11"/>
       <c r="M22" s="11"/>
-      <c r="N22" s="10"/>
+      <c r="N22" s="11"/>
       <c r="O22" s="10"/>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P22" s="10"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B23" s="10"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11"/>
-      <c r="E23" s="10"/>
+      <c r="E23" s="11"/>
       <c r="F23" s="10"/>
       <c r="G23" s="10"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="11"/>
       <c r="J23" s="10"/>
-      <c r="K23" s="13">
+      <c r="K23" s="10"/>
+      <c r="L23" s="13">
         <v>5</v>
       </c>
-      <c r="L23" s="11"/>
       <c r="M23" s="11"/>
-      <c r="N23" s="10"/>
+      <c r="N23" s="11"/>
       <c r="O23" s="10"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P23" s="10"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="11"/>
       <c r="D24" s="11"/>
-      <c r="E24" s="10"/>
+      <c r="E24" s="11"/>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="11"/>
       <c r="J24" s="10"/>
-      <c r="K24" s="13">
+      <c r="K24" s="10"/>
+      <c r="L24" s="13">
         <v>5</v>
       </c>
-      <c r="L24" s="11"/>
       <c r="M24" s="11"/>
-      <c r="N24" s="10"/>
+      <c r="N24" s="11"/>
       <c r="O24" s="10"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P24" s="10"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A25" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B25" s="10"/>
       <c r="C25" s="11"/>
       <c r="D25" s="11"/>
-      <c r="E25" s="10"/>
+      <c r="E25" s="11"/>
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="11"/>
       <c r="J25" s="10"/>
-      <c r="K25" s="13">
+      <c r="K25" s="10"/>
+      <c r="L25" s="13">
         <v>5</v>
       </c>
-      <c r="L25" s="11"/>
       <c r="M25" s="11"/>
-      <c r="N25" s="10"/>
+      <c r="N25" s="11"/>
       <c r="O25" s="10"/>
-      <c r="P25" s="6"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P25" s="10"/>
+      <c r="Q25" s="6"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A26" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B26" s="10"/>
       <c r="C26" s="11"/>
       <c r="D26" s="11"/>
-      <c r="E26" s="10"/>
+      <c r="E26" s="11"/>
       <c r="F26" s="10"/>
       <c r="G26" s="10"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="11"/>
       <c r="J26" s="10"/>
-      <c r="K26" s="13">
+      <c r="K26" s="10"/>
+      <c r="L26" s="13">
         <v>6</v>
       </c>
-      <c r="L26" s="11"/>
       <c r="M26" s="11"/>
-      <c r="N26" s="10"/>
+      <c r="N26" s="11"/>
       <c r="O26" s="10"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P26" s="10"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B27" s="10"/>
       <c r="C27" s="11"/>
       <c r="D27" s="11"/>
-      <c r="E27" s="10"/>
+      <c r="E27" s="11"/>
       <c r="F27" s="10"/>
       <c r="G27" s="10"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="11"/>
       <c r="J27" s="10"/>
-      <c r="K27" s="2">
+      <c r="K27" s="10"/>
+      <c r="L27" s="2">
         <v>6</v>
       </c>
-      <c r="L27" s="11"/>
       <c r="M27" s="11"/>
-      <c r="N27" s="10"/>
+      <c r="N27" s="11"/>
       <c r="O27" s="10"/>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P27" s="10"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
         <v>20</v>
       </c>
       <c r="B28" s="10"/>
       <c r="C28" s="11"/>
       <c r="D28" s="11"/>
-      <c r="E28" s="10"/>
+      <c r="E28" s="11"/>
       <c r="F28" s="10"/>
       <c r="G28" s="10"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="11"/>
       <c r="J28" s="10"/>
-      <c r="K28" s="2">
+      <c r="K28" s="10"/>
+      <c r="L28" s="2">
         <v>6</v>
       </c>
-      <c r="L28" s="11"/>
       <c r="M28" s="11"/>
-      <c r="N28" s="10"/>
+      <c r="N28" s="11"/>
       <c r="O28" s="10"/>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P28" s="10"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B29" s="10"/>
       <c r="C29" s="11"/>
       <c r="D29" s="11"/>
-      <c r="E29" s="10"/>
+      <c r="E29" s="11"/>
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="11"/>
       <c r="J29" s="10"/>
-      <c r="K29" s="2">
+      <c r="K29" s="10"/>
+      <c r="L29" s="2">
         <v>4</v>
       </c>
-      <c r="L29" s="11"/>
       <c r="M29" s="11"/>
-      <c r="N29" s="10"/>
+      <c r="N29" s="11"/>
       <c r="O29" s="10"/>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P29" s="10"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A30" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B30" s="10"/>
       <c r="C30" s="11"/>
       <c r="D30" s="11"/>
-      <c r="E30" s="10"/>
+      <c r="E30" s="11"/>
       <c r="F30" s="10"/>
       <c r="G30" s="10"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="11"/>
       <c r="J30" s="10"/>
-      <c r="K30" s="2">
+      <c r="K30" s="10"/>
+      <c r="L30" s="2">
         <v>5</v>
       </c>
-      <c r="L30" s="11"/>
       <c r="M30" s="11"/>
-      <c r="N30" s="10"/>
+      <c r="N30" s="11"/>
       <c r="O30" s="10"/>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P30" s="10"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B31" s="10"/>
       <c r="C31" s="11"/>
       <c r="D31" s="11"/>
-      <c r="E31" s="10"/>
+      <c r="E31" s="11"/>
       <c r="F31" s="10"/>
       <c r="G31" s="10"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="11"/>
       <c r="J31" s="10"/>
-      <c r="K31" s="2">
+      <c r="K31" s="10"/>
+      <c r="L31" s="2">
         <v>5</v>
       </c>
-      <c r="L31" s="11"/>
       <c r="M31" s="11"/>
-      <c r="N31" s="10"/>
+      <c r="N31" s="11"/>
       <c r="O31" s="10"/>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="P31" s="10"/>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A32" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B32" s="10"/>
       <c r="C32" s="11"/>
       <c r="D32" s="11"/>
-      <c r="E32" s="10"/>
+      <c r="E32" s="11"/>
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="11"/>
       <c r="J32" s="10"/>
-      <c r="K32" s="2">
+      <c r="K32" s="10"/>
+      <c r="L32" s="2">
         <v>5</v>
       </c>
-      <c r="L32" s="11"/>
       <c r="M32" s="11"/>
-      <c r="N32" s="10"/>
+      <c r="N32" s="11"/>
       <c r="O32" s="10"/>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P32" s="10"/>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A33" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B33" s="10"/>
       <c r="C33" s="11"/>
       <c r="D33" s="11"/>
-      <c r="E33" s="10"/>
+      <c r="E33" s="11"/>
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="11"/>
       <c r="J33" s="10"/>
-      <c r="K33" s="2">
+      <c r="K33" s="10"/>
+      <c r="L33" s="2">
         <v>5</v>
       </c>
-      <c r="L33" s="11"/>
       <c r="M33" s="11"/>
-      <c r="N33" s="10"/>
+      <c r="N33" s="11"/>
       <c r="O33" s="10"/>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P33" s="10"/>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B34" s="10"/>
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
-      <c r="E34" s="10"/>
+      <c r="E34" s="11"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="11"/>
       <c r="J34" s="10"/>
-      <c r="K34" s="2">
+      <c r="K34" s="10"/>
+      <c r="L34" s="2">
         <v>5</v>
       </c>
-      <c r="L34" s="11"/>
       <c r="M34" s="11"/>
-      <c r="N34" s="10"/>
+      <c r="N34" s="11"/>
       <c r="O34" s="10"/>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P34" s="10"/>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="10"/>
       <c r="C35" s="11"/>
       <c r="D35" s="11"/>
-      <c r="E35" s="10"/>
+      <c r="E35" s="11"/>
       <c r="F35" s="10"/>
       <c r="G35" s="10"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="11"/>
       <c r="J35" s="10"/>
-      <c r="K35" s="2">
+      <c r="K35" s="10"/>
+      <c r="L35" s="2">
         <v>5</v>
       </c>
-      <c r="L35" s="11"/>
       <c r="M35" s="11"/>
-      <c r="N35" s="10"/>
+      <c r="N35" s="11"/>
       <c r="O35" s="10"/>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P35" s="10"/>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A36" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B36" s="10"/>
       <c r="C36" s="11"/>
       <c r="D36" s="11"/>
-      <c r="E36" s="10"/>
+      <c r="E36" s="11"/>
       <c r="F36" s="10"/>
       <c r="G36" s="10"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="11"/>
       <c r="J36" s="10"/>
-      <c r="K36" s="2">
+      <c r="K36" s="10"/>
+      <c r="L36" s="2">
         <v>5</v>
       </c>
-      <c r="L36" s="11"/>
       <c r="M36" s="11"/>
-      <c r="N36" s="10"/>
+      <c r="N36" s="11"/>
       <c r="O36" s="10"/>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P36" s="10"/>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A37" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B37" s="10"/>
       <c r="C37" s="11"/>
       <c r="D37" s="11"/>
-      <c r="E37" s="10"/>
+      <c r="E37" s="11"/>
       <c r="F37" s="10"/>
       <c r="G37" s="10"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="11"/>
       <c r="J37" s="10"/>
-      <c r="K37" s="2">
+      <c r="K37" s="10"/>
+      <c r="L37" s="2">
         <v>5</v>
       </c>
-      <c r="L37" s="11"/>
       <c r="M37" s="11"/>
-      <c r="N37" s="10"/>
+      <c r="N37" s="11"/>
       <c r="O37" s="10"/>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P37" s="10"/>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A38" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B38" s="10"/>
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
-      <c r="E38" s="10"/>
+      <c r="E38" s="11"/>
       <c r="F38" s="10"/>
       <c r="G38" s="10"/>
-      <c r="H38" s="11"/>
-      <c r="I38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="11"/>
       <c r="J38" s="10"/>
-      <c r="K38" s="2">
+      <c r="K38" s="10"/>
+      <c r="L38" s="2">
         <v>6</v>
       </c>
-      <c r="L38" s="11"/>
       <c r="M38" s="11"/>
-      <c r="N38" s="10"/>
+      <c r="N38" s="11"/>
       <c r="O38" s="10"/>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P38" s="10"/>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A39" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B39" s="10"/>
       <c r="C39" s="11"/>
       <c r="D39" s="11"/>
-      <c r="E39" s="10"/>
+      <c r="E39" s="11"/>
       <c r="F39" s="10"/>
       <c r="G39" s="10"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="11"/>
       <c r="J39" s="10"/>
-      <c r="K39" s="2">
+      <c r="K39" s="10"/>
+      <c r="L39" s="2">
         <v>6</v>
       </c>
-      <c r="L39" s="11"/>
       <c r="M39" s="11"/>
-      <c r="N39" s="10"/>
+      <c r="N39" s="11"/>
       <c r="O39" s="10"/>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P39" s="10"/>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A40" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B40" s="10"/>
       <c r="C40" s="11"/>
       <c r="D40" s="11"/>
-      <c r="E40" s="10"/>
+      <c r="E40" s="11"/>
       <c r="F40" s="10"/>
       <c r="G40" s="10"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="11"/>
       <c r="J40" s="10"/>
-      <c r="K40" s="2">
+      <c r="K40" s="10"/>
+      <c r="L40" s="2">
         <v>6</v>
       </c>
-      <c r="L40" s="11"/>
       <c r="M40" s="11"/>
-      <c r="N40" s="10"/>
+      <c r="N40" s="11"/>
       <c r="O40" s="10"/>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P40" s="10"/>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B41" s="10"/>
       <c r="C41" s="11"/>
       <c r="D41" s="11"/>
-      <c r="E41" s="10"/>
+      <c r="E41" s="11"/>
       <c r="F41" s="10"/>
       <c r="G41" s="10"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="11"/>
       <c r="J41" s="10"/>
-      <c r="K41" s="2">
+      <c r="K41" s="10"/>
+      <c r="L41" s="2">
         <v>6</v>
       </c>
-      <c r="L41" s="11"/>
       <c r="M41" s="11"/>
-      <c r="N41" s="10"/>
+      <c r="N41" s="11"/>
       <c r="O41" s="10"/>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P41" s="10"/>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A42" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B42" s="10"/>
       <c r="C42" s="11"/>
       <c r="D42" s="11"/>
-      <c r="E42" s="10"/>
+      <c r="E42" s="11"/>
       <c r="F42" s="10"/>
       <c r="G42" s="10"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="I42" s="11"/>
       <c r="J42" s="10"/>
-      <c r="K42" s="2">
+      <c r="K42" s="10"/>
+      <c r="L42" s="2">
         <v>6</v>
       </c>
-      <c r="L42" s="11"/>
       <c r="M42" s="11"/>
-      <c r="N42" s="10"/>
+      <c r="N42" s="11"/>
       <c r="O42" s="10"/>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P42" s="10"/>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B43" s="10"/>
       <c r="C43" s="11"/>
       <c r="D43" s="11"/>
-      <c r="E43" s="10"/>
+      <c r="E43" s="11"/>
       <c r="F43" s="10"/>
       <c r="G43" s="10"/>
-      <c r="H43" s="11"/>
-      <c r="I43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="11"/>
       <c r="J43" s="10"/>
-      <c r="K43" s="2">
+      <c r="K43" s="10"/>
+      <c r="L43" s="2">
         <v>6</v>
       </c>
-      <c r="L43" s="11"/>
       <c r="M43" s="11"/>
-      <c r="N43" s="10"/>
+      <c r="N43" s="11"/>
       <c r="O43" s="10"/>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P43" s="10"/>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A44" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B44" s="10"/>
       <c r="C44" s="11"/>
       <c r="D44" s="11"/>
-      <c r="E44" s="10"/>
+      <c r="E44" s="11"/>
       <c r="F44" s="10"/>
       <c r="G44" s="10"/>
-      <c r="H44" s="11"/>
-      <c r="I44" s="10"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="11"/>
       <c r="J44" s="10"/>
-      <c r="K44" s="2">
+      <c r="K44" s="10"/>
+      <c r="L44" s="2">
         <v>6</v>
       </c>
-      <c r="L44" s="11"/>
       <c r="M44" s="11"/>
-      <c r="N44" s="10"/>
+      <c r="N44" s="11"/>
       <c r="O44" s="10"/>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P44" s="10"/>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A45" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B45" s="10"/>
       <c r="C45" s="11"/>
       <c r="D45" s="11"/>
-      <c r="E45" s="10"/>
+      <c r="E45" s="11"/>
       <c r="F45" s="10"/>
       <c r="G45" s="10"/>
-      <c r="H45" s="11"/>
-      <c r="I45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="11"/>
       <c r="J45" s="10"/>
-      <c r="K45" s="2">
+      <c r="K45" s="10"/>
+      <c r="L45" s="2">
         <v>4</v>
       </c>
-      <c r="L45" s="11"/>
       <c r="M45" s="11"/>
-      <c r="N45" s="10"/>
+      <c r="N45" s="11"/>
       <c r="O45" s="10"/>
-    </row>
-    <row r="46" spans="1:15" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P45" s="10"/>
+    </row>
+    <row r="46" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B46" s="10"/>
       <c r="C46" s="11"/>
       <c r="D46" s="11"/>
-      <c r="E46" s="10"/>
+      <c r="E46" s="11"/>
       <c r="F46" s="10"/>
       <c r="G46" s="10"/>
-      <c r="H46" s="11"/>
-      <c r="I46" s="10"/>
+      <c r="H46" s="10"/>
+      <c r="I46" s="11"/>
       <c r="J46" s="10"/>
-      <c r="K46" s="2">
+      <c r="K46" s="10"/>
+      <c r="L46" s="2">
         <v>5</v>
       </c>
-      <c r="L46" s="11"/>
       <c r="M46" s="11"/>
-      <c r="N46" s="10"/>
+      <c r="N46" s="11"/>
       <c r="O46" s="10"/>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P46" s="10"/>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B47" s="10"/>
       <c r="C47" s="11"/>
       <c r="D47" s="11"/>
-      <c r="E47" s="10"/>
+      <c r="E47" s="11"/>
       <c r="F47" s="10"/>
       <c r="G47" s="10"/>
-      <c r="H47" s="11"/>
-      <c r="I47" s="10"/>
+      <c r="H47" s="10"/>
+      <c r="I47" s="11"/>
       <c r="J47" s="10"/>
-      <c r="K47" s="2">
+      <c r="K47" s="10"/>
+      <c r="L47" s="2">
         <v>5</v>
       </c>
-      <c r="L47" s="11"/>
       <c r="M47" s="11"/>
-      <c r="N47" s="10"/>
+      <c r="N47" s="11"/>
       <c r="O47" s="10"/>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P47" s="10"/>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A48" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B48" s="10"/>
       <c r="C48" s="11"/>
       <c r="D48" s="11"/>
-      <c r="E48" s="10"/>
+      <c r="E48" s="11"/>
       <c r="F48" s="10"/>
       <c r="G48" s="10"/>
-      <c r="H48" s="11"/>
-      <c r="I48" s="10"/>
+      <c r="H48" s="10"/>
+      <c r="I48" s="11"/>
       <c r="J48" s="10"/>
-      <c r="K48" s="2">
+      <c r="K48" s="10"/>
+      <c r="L48" s="2">
         <v>5</v>
       </c>
-      <c r="L48" s="11"/>
       <c r="M48" s="11"/>
-      <c r="N48" s="10"/>
+      <c r="N48" s="11"/>
       <c r="O48" s="10"/>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P48" s="10"/>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A49" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B49" s="10"/>
       <c r="C49" s="11"/>
       <c r="D49" s="11"/>
-      <c r="E49" s="10"/>
+      <c r="E49" s="11"/>
       <c r="F49" s="10"/>
       <c r="G49" s="10"/>
-      <c r="H49" s="11"/>
-      <c r="I49" s="10"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="11"/>
       <c r="J49" s="10"/>
-      <c r="K49" s="2">
+      <c r="K49" s="10"/>
+      <c r="L49" s="2">
         <v>5</v>
       </c>
-      <c r="L49" s="11"/>
       <c r="M49" s="11"/>
-      <c r="N49" s="10"/>
+      <c r="N49" s="11"/>
       <c r="O49" s="10"/>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P49" s="10"/>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A50" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B50" s="10"/>
       <c r="C50" s="11"/>
       <c r="D50" s="11"/>
-      <c r="E50" s="10"/>
+      <c r="E50" s="11"/>
       <c r="F50" s="10"/>
       <c r="G50" s="10"/>
-      <c r="H50" s="11"/>
-      <c r="I50" s="10"/>
+      <c r="H50" s="10"/>
+      <c r="I50" s="11"/>
       <c r="J50" s="10"/>
-      <c r="K50" s="2">
+      <c r="K50" s="10"/>
+      <c r="L50" s="2">
         <v>6</v>
       </c>
-      <c r="L50" s="11"/>
       <c r="M50" s="11"/>
-      <c r="N50" s="10"/>
+      <c r="N50" s="11"/>
       <c r="O50" s="10"/>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P50" s="10"/>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A51" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B51" s="10"/>
       <c r="C51" s="11"/>
       <c r="D51" s="11"/>
-      <c r="E51" s="10"/>
+      <c r="E51" s="11"/>
       <c r="F51" s="10"/>
       <c r="G51" s="10"/>
-      <c r="H51" s="11"/>
-      <c r="I51" s="10"/>
+      <c r="H51" s="10"/>
+      <c r="I51" s="11"/>
       <c r="J51" s="10"/>
-      <c r="K51" s="2">
+      <c r="K51" s="10"/>
+      <c r="L51" s="2">
         <v>6</v>
       </c>
-      <c r="L51" s="11"/>
       <c r="M51" s="11"/>
-      <c r="N51" s="10"/>
+      <c r="N51" s="11"/>
       <c r="O51" s="10"/>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P51" s="10"/>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A52" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B52" s="10"/>
       <c r="C52" s="11"/>
       <c r="D52" s="11"/>
-      <c r="E52" s="10"/>
+      <c r="E52" s="11"/>
       <c r="F52" s="10"/>
       <c r="G52" s="10"/>
-      <c r="H52" s="11"/>
-      <c r="I52" s="10"/>
+      <c r="H52" s="10"/>
+      <c r="I52" s="11"/>
       <c r="J52" s="10"/>
-      <c r="K52" s="2">
+      <c r="K52" s="10"/>
+      <c r="L52" s="2">
         <v>6</v>
       </c>
-      <c r="L52" s="11"/>
       <c r="M52" s="11"/>
-      <c r="N52" s="10"/>
+      <c r="N52" s="11"/>
       <c r="O52" s="10"/>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P52" s="10"/>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A53" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B53" s="10"/>
       <c r="C53" s="11"/>
       <c r="D53" s="11"/>
-      <c r="E53" s="10"/>
+      <c r="E53" s="11"/>
       <c r="F53" s="10"/>
       <c r="G53" s="10"/>
-      <c r="H53" s="11"/>
-      <c r="I53" s="10"/>
+      <c r="H53" s="10"/>
+      <c r="I53" s="11"/>
       <c r="J53" s="10"/>
-      <c r="K53" s="2">
+      <c r="K53" s="10"/>
+      <c r="L53" s="2">
         <v>5</v>
       </c>
-      <c r="L53" s="11"/>
       <c r="M53" s="11"/>
-      <c r="N53" s="10"/>
+      <c r="N53" s="11"/>
       <c r="O53" s="10"/>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P53" s="10"/>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A54" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B54" s="10"/>
       <c r="C54" s="11"/>
       <c r="D54" s="11"/>
-      <c r="E54" s="10"/>
+      <c r="E54" s="11"/>
       <c r="F54" s="10"/>
       <c r="G54" s="10"/>
-      <c r="H54" s="11"/>
-      <c r="I54" s="10"/>
+      <c r="H54" s="10"/>
+      <c r="I54" s="11"/>
       <c r="J54" s="10"/>
-      <c r="K54" s="2">
+      <c r="K54" s="10"/>
+      <c r="L54" s="2">
         <v>6</v>
       </c>
-      <c r="L54" s="11"/>
       <c r="M54" s="11"/>
-      <c r="N54" s="10"/>
+      <c r="N54" s="11"/>
       <c r="O54" s="10"/>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P54" s="10"/>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A55" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B55" s="10"/>
       <c r="C55" s="11"/>
       <c r="D55" s="11"/>
-      <c r="E55" s="10"/>
+      <c r="E55" s="11"/>
       <c r="F55" s="10"/>
       <c r="G55" s="10"/>
-      <c r="H55" s="11"/>
-      <c r="I55" s="10"/>
+      <c r="H55" s="10"/>
+      <c r="I55" s="11"/>
       <c r="J55" s="10"/>
-      <c r="K55" s="2">
+      <c r="K55" s="10"/>
+      <c r="L55" s="2">
         <v>6</v>
       </c>
-      <c r="L55" s="11"/>
       <c r="M55" s="11"/>
-      <c r="N55" s="10"/>
+      <c r="N55" s="11"/>
       <c r="O55" s="10"/>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P55" s="10"/>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A56" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B56" s="10"/>
       <c r="C56" s="11"/>
       <c r="D56" s="11"/>
-      <c r="E56" s="10"/>
+      <c r="E56" s="11"/>
       <c r="F56" s="10"/>
       <c r="G56" s="10"/>
-      <c r="H56" s="11"/>
-      <c r="I56" s="10"/>
+      <c r="H56" s="10"/>
+      <c r="I56" s="11"/>
       <c r="J56" s="10"/>
-      <c r="K56" s="2">
+      <c r="K56" s="10"/>
+      <c r="L56" s="2">
         <v>6</v>
       </c>
-      <c r="L56" s="11"/>
       <c r="M56" s="11"/>
-      <c r="N56" s="10"/>
+      <c r="N56" s="11"/>
       <c r="O56" s="10"/>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P56" s="10"/>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B57" s="10"/>
       <c r="C57" s="11"/>
       <c r="D57" s="11"/>
-      <c r="E57" s="10"/>
+      <c r="E57" s="11"/>
       <c r="F57" s="10"/>
       <c r="G57" s="10"/>
-      <c r="H57" s="11"/>
-      <c r="I57" s="10"/>
+      <c r="H57" s="10"/>
+      <c r="I57" s="11"/>
       <c r="J57" s="10"/>
-      <c r="K57" s="2">
+      <c r="K57" s="10"/>
+      <c r="L57" s="2">
         <v>6</v>
       </c>
-      <c r="L57" s="11"/>
       <c r="M57" s="11"/>
-      <c r="N57" s="10"/>
+      <c r="N57" s="11"/>
       <c r="O57" s="10"/>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P57" s="10"/>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A58" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B58" s="10"/>
       <c r="C58" s="11"/>
       <c r="D58" s="11"/>
-      <c r="E58" s="10"/>
+      <c r="E58" s="11"/>
       <c r="F58" s="10"/>
       <c r="G58" s="10"/>
-      <c r="H58" s="11"/>
-      <c r="I58" s="10"/>
+      <c r="H58" s="10"/>
+      <c r="I58" s="11"/>
       <c r="J58" s="10"/>
-      <c r="K58" s="2">
+      <c r="K58" s="10"/>
+      <c r="L58" s="2">
         <v>6</v>
       </c>
-      <c r="L58" s="11"/>
       <c r="M58" s="11"/>
-      <c r="N58" s="10"/>
+      <c r="N58" s="11"/>
       <c r="O58" s="10"/>
+      <c r="P58" s="10"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:O5 A6:J8 L6:O8">
-    <cfRule type="containsBlanks" dxfId="3" priority="4">
+  <conditionalFormatting sqref="A2:P5 M6:P8 A6:K58">
+    <cfRule type="expression" dxfId="3" priority="3">
+      <formula>COUNTA($A2:$P2)=COLUMNS($A2:$P2)</formula>
+    </cfRule>
+    <cfRule type="containsBlanks" dxfId="2" priority="4">
       <formula>LEN(TRIM(A2))=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="3">
-      <formula>COUNTA($A2:$O2)=COLUMNS($A2:$O2)</formula>
-    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L9:O58 A9:J58">
+  <conditionalFormatting sqref="M9:P58">
     <cfRule type="expression" dxfId="1" priority="1">
-      <formula>COUNTA($A9:$O9)=COLUMNS($A9:$O9)</formula>
+      <formula>COUNTA($A9:$P9)=COLUMNS($A9:$P9)</formula>
     </cfRule>
     <cfRule type="containsBlanks" dxfId="0" priority="2">
-      <formula>LEN(TRIM(A9))=0</formula>
+      <formula>LEN(TRIM(M9))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q8 C2:C58">
-      <formula1>$Q$1:$Q$8</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R8 C2:C58">
+      <formula1>$R$1:$R$8</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H58">
-      <formula1>$S$2:$S$8</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I58">
+      <formula1>$T$2:$T$8</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A58">
-      <formula1>$P$1:$P$6</formula1>
+      <formula1>$Q$1:$Q$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="K3" twoDigitTextYear="1"/>
+    <ignoredError sqref="L3" twoDigitTextYear="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Correct rally 4 group 2
</commit_message>
<xml_diff>
--- a/Rallies.xlsx
+++ b/Rallies.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="81">
   <si>
     <t>Year</t>
   </si>
@@ -235,10 +235,28 @@
     <t>After their win in the grueling &lt;b&gt;London-Mexico World Cup Rally&lt;/b&gt;, &lt;b&gt;Hannu Mikkola&lt;/b&gt; and the exceptional navigator &lt;b&gt;Gunnar Palm&lt;/b&gt; brought their Ford Escort twin cam to Finland. With its engine originally developped for the Lotus Elan and its lights body shell the Escort proved to be a solid contender for the rougher rallies.</t>
   </si>
   <si>
-    <t>Morning, Rain, Afternoon, Morning</t>
-  </si>
-  <si>
-    <t>0, 5, 6, 8</t>
+    <t>Rally Sanremo</t>
+  </si>
+  <si>
+    <t>5-9 March</t>
+  </si>
+  <si>
+    <t>Harry Källström</t>
+  </si>
+  <si>
+    <t>Sunset, Afternoon, Sunset, Afternoon</t>
+  </si>
+  <si>
+    <t>2, 6, 10, 0</t>
+  </si>
+  <si>
+    <t>Morning, Afternoon, Morning, Sunset, Rain</t>
+  </si>
+  <si>
+    <t>0, 5, 6, 8 , 2</t>
+  </si>
+  <si>
+    <t>Nicknamed "Sputnik" because of how fast his career took off, driver and later actorn &lt;b&gt;Harry Källström&lt;/b&gt; took the wheel of a Lancia Fulvia with his copilot &lt;b&gt;Häggbom Gunnar&lt;/b&gt; to win the &lt;b&gt;Sanremo Rally&lt;/b&gt; as well as the &lt;b&gt;Spanish RACE Rally&lt;/b&gt; and &lt;b&gt;British RAC Rally&lt;/b&gt; that year, earning their first European champions title.</t>
   </si>
 </sst>
 </file>
@@ -357,7 +375,21 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -982,43 +1014,43 @@
         <v>12</v>
       </c>
       <c r="B5" s="9">
+        <v>1969</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="H5" s="9">
         <v>1970</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="I5" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="J5" s="9">
         <v>3</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="9">
-        <v>1966</v>
-      </c>
-      <c r="I5" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="J5" s="9">
-        <v>1</v>
-      </c>
       <c r="K5" s="9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="O5" s="9" t="s">
         <v>63</v>
@@ -1048,23 +1080,51 @@
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
+      <c r="B6" s="9">
+        <v>1970</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="9">
+        <v>1966</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" s="9">
+        <v>1</v>
+      </c>
+      <c r="K6" s="9">
+        <v>2</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="N6" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="O6" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="P6" s="9" t="s">
+        <v>63</v>
+      </c>
       <c r="Q6" s="11" t="s">
         <v>23</v>
       </c>
@@ -2356,20 +2416,28 @@
       <c r="P58" s="9"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:P5 M6:P8 A6:K58">
-    <cfRule type="expression" dxfId="3" priority="3">
+  <conditionalFormatting sqref="A2:P5 M7:P8 A7:K58">
+    <cfRule type="expression" dxfId="5" priority="5">
       <formula>COUNTA($A2:$P2)=COLUMNS($A2:$P2)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="2" priority="4">
+    <cfRule type="containsBlanks" dxfId="4" priority="6">
       <formula>LEN(TRIM(A2))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M9:P58">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>COUNTA($A9:$P9)=COLUMNS($A9:$P9)</formula>
     </cfRule>
+    <cfRule type="containsBlanks" dxfId="2" priority="4">
+      <formula>LEN(TRIM(M9))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A6:P6">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>COUNTA($A6:$P6)=COLUMNS($A6:$P6)</formula>
+    </cfRule>
     <cfRule type="containsBlanks" dxfId="0" priority="2">
-      <formula>LEN(TRIM(M9))=0</formula>
+      <formula>LEN(TRIM(A6))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">

</xml_diff>

<commit_message>
Add rally 6 group 2
</commit_message>
<xml_diff>
--- a/Rallies.xlsx
+++ b/Rallies.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="85">
   <si>
     <t>Year</t>
   </si>
@@ -184,15 +184,6 @@
     <t>22-26 February</t>
   </si>
   <si>
-    <t>// 2</t>
-  </si>
-  <si>
-    <t>// 5</t>
-  </si>
-  <si>
-    <t>// 6</t>
-  </si>
-  <si>
     <t>Fog, Afternoon, Sunset</t>
   </si>
   <si>
@@ -257,6 +248,27 @@
   </si>
   <si>
     <t>Nicknamed "Sputnik" because of how fast his career took off, driver and later actorn &lt;b&gt;Harry Källström&lt;/b&gt; took the wheel of a Lancia Fulvia with his copilot &lt;b&gt;Häggbom Gunnar&lt;/b&gt; to win the &lt;b&gt;Sanremo Rally&lt;/b&gt; as well as the &lt;b&gt;Spanish RACE Rally&lt;/b&gt; and &lt;b&gt;British RAC Rally&lt;/b&gt; that year, earning their first European champions title.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jean-Claude Andruet </t>
+  </si>
+  <si>
+    <t>1-3 October</t>
+  </si>
+  <si>
+    <t>Austria</t>
+  </si>
+  <si>
+    <t>Rally Munich-Vienne-Budapest</t>
+  </si>
+  <si>
+    <t>1, 8, 10, 5, 7</t>
+  </si>
+  <si>
+    <t>After dominating in the french rallies, &lt;b&gt;Jean-Claude Andruet&lt;/b&gt; wildly swong his &lt;b&gt;Alpine A110&lt;/b&gt; with &lt;b&gt;Michèle Veron&lt;/b&gt; as copilot in this rally spanning between Germany, Austria and Hungary. The battle with Fords and Porsches was fierce but they won the French and European rally championships titles.</t>
+  </si>
+  <si>
+    <t>Rain, Morning, Rain, Sunset, Fog</t>
   </si>
 </sst>
 </file>
@@ -327,12 +339,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -344,38 +353,74 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="12">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -720,15 +765,16 @@
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="7" style="1" customWidth="1"/>
-    <col min="3" max="4" width="9" style="4" customWidth="1"/>
+    <col min="3" max="4" width="9" style="3" customWidth="1"/>
     <col min="5" max="5" width="15.81640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.81640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.7265625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="19" style="1" customWidth="1"/>
     <col min="8" max="8" width="12.1796875" style="1" customWidth="1"/>
     <col min="9" max="9" width="14.54296875" style="1" customWidth="1"/>
     <col min="10" max="10" width="7.1796875" style="1" customWidth="1"/>
     <col min="11" max="11" width="12.26953125" style="1" customWidth="1"/>
-    <col min="12" max="13" width="9.81640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="10.81640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="9.81640625" style="1" customWidth="1"/>
     <col min="14" max="14" width="62" style="1" customWidth="1"/>
     <col min="15" max="16" width="8.453125" style="1" customWidth="1"/>
     <col min="17" max="18" width="9.1796875" style="1" customWidth="1"/>
@@ -739,74 +785,74 @@
     <col min="23" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="3" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:25" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="E1" s="5" t="s">
+      <c r="D1" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="G1" s="5" t="s">
+      <c r="F1" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="O1" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q1" s="11" t="s">
+      <c r="O1" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="R1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="S1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="T1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="U1" s="7" t="s">
+      <c r="U1" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="V1" s="7"/>
-      <c r="W1" s="7"/>
-      <c r="X1" s="7"/>
-      <c r="Y1" s="7"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
+      <c r="X1" s="5"/>
+      <c r="Y1" s="5"/>
     </row>
     <row r="2" spans="1:25" ht="78" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
@@ -815,13 +861,13 @@
       <c r="B2" s="9">
         <v>1966</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="9" t="s">
         <v>4</v>
       </c>
       <c r="F2" s="9" t="s">
@@ -833,7 +879,7 @@
       <c r="H2" s="9">
         <v>1966</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="9" t="s">
         <v>48</v>
       </c>
       <c r="J2" s="9">
@@ -845,35 +891,35 @@
       <c r="L2" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="M2" s="11" t="s">
+      <c r="M2" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="N2" s="9" t="s">
         <v>31</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="P2" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q2" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="R2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="S2" s="8" t="s">
+      <c r="S2" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
-      <c r="Y2" s="4"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="3"/>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+      <c r="Y2" s="3"/>
     </row>
     <row r="3" spans="1:25" ht="74.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
@@ -882,13 +928,13 @@
       <c r="B3" s="9">
         <v>1967</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="E3" s="10" t="s">
+      <c r="D3" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>6</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -900,7 +946,7 @@
       <c r="H3" s="9">
         <v>1967</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="9" t="s">
         <v>47</v>
       </c>
       <c r="J3" s="9">
@@ -910,37 +956,37 @@
         <v>0</v>
       </c>
       <c r="L3" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="O3" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="M3" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="N3" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="O3" s="9" t="s">
-        <v>63</v>
-      </c>
       <c r="P3" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q3" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="R3" s="11" t="s">
+      <c r="R3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="S3" s="8" t="s">
+      <c r="S3" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="T3" s="4" t="s">
+      <c r="T3" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="4"/>
-      <c r="Y3" s="4"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
     </row>
     <row r="4" spans="1:25" ht="81.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
@@ -949,17 +995,17 @@
       <c r="B4" s="9">
         <v>1968</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E4" s="10" t="s">
+      <c r="D4" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>10</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>9</v>
@@ -967,7 +1013,7 @@
       <c r="H4" s="9">
         <v>1969</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>46</v>
       </c>
       <c r="J4" s="9">
@@ -977,37 +1023,37 @@
         <v>0</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="M4" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="N4" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="M4" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="N4" s="9" t="s">
         <v>51</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="P4" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q4" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q4" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="R4" s="11" t="s">
+      <c r="R4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="S4" s="8" t="s">
+      <c r="S4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="T4" s="4" t="s">
+      <c r="T4" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="U4" s="4"/>
-      <c r="V4" s="4"/>
-      <c r="W4" s="4"/>
-      <c r="X4" s="4"/>
-      <c r="Y4" s="4"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
     </row>
     <row r="5" spans="1:25" ht="91" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
@@ -1016,25 +1062,25 @@
       <c r="B5" s="9">
         <v>1969</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>73</v>
+      <c r="D5" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>70</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H5" s="9">
         <v>1970</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="I5" s="9" t="s">
         <v>49</v>
       </c>
       <c r="J5" s="9">
@@ -1044,37 +1090,37 @@
         <v>0</v>
       </c>
       <c r="L5" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="N5" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="M5" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="N5" s="10" t="s">
-        <v>80</v>
-      </c>
       <c r="O5" s="9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="P5" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q5" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q5" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="R5" s="11" t="s">
+      <c r="R5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="S5" s="8" t="s">
+      <c r="S5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="T5" s="4" t="s">
+      <c r="T5" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4"/>
-      <c r="X5" s="4"/>
-      <c r="Y5" s="4"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
     </row>
     <row r="6" spans="1:25" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
@@ -1083,17 +1129,17 @@
       <c r="B6" s="9">
         <v>1970</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="9" t="s">
         <v>4</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="G6" s="9" t="s">
         <v>11</v>
@@ -1101,7 +1147,7 @@
       <c r="H6" s="9">
         <v>1966</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="9" t="s">
         <v>43</v>
       </c>
       <c r="J6" s="9">
@@ -1111,1333 +1157,1539 @@
         <v>2</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="M6" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="N6" s="10" t="s">
-        <v>72</v>
+        <v>76</v>
+      </c>
+      <c r="M6" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="N6" s="9" t="s">
+        <v>69</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="P6" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q6" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q6" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="R6" s="11" t="s">
+      <c r="R6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="S6" s="8" t="s">
+      <c r="S6" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="T6" s="4" t="s">
+      <c r="T6" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="U6" s="4"/>
-      <c r="V6" s="4"/>
-      <c r="W6" s="4"/>
-      <c r="X6" s="4"/>
-      <c r="Y6" s="4"/>
-    </row>
-    <row r="7" spans="1:25" ht="29" x14ac:dyDescent="0.35">
+      <c r="U6" s="10"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="3"/>
+      <c r="X6" s="3"/>
+      <c r="Y6" s="3"/>
+    </row>
+    <row r="7" spans="1:25" ht="84" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="4"/>
-      <c r="R7" s="11" t="s">
+      <c r="B7" s="9">
+        <v>1970</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="H7" s="9">
+        <v>1977</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" s="9">
+        <v>5</v>
+      </c>
+      <c r="K7" s="9">
+        <v>6</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="O7" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="P7" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q7" s="10"/>
+      <c r="R7" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="S7" s="8" t="s">
+      <c r="S7" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="T7" s="4" t="s">
+      <c r="T7" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="U7" s="4"/>
-      <c r="V7" s="4"/>
-      <c r="W7" s="4"/>
-      <c r="X7" s="4"/>
-      <c r="Y7" s="4"/>
+      <c r="U7" s="10"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="3"/>
+      <c r="X7" s="3"/>
+      <c r="Y7" s="3"/>
     </row>
     <row r="8" spans="1:25" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B8" s="9"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
       <c r="F8" s="9"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9"/>
-      <c r="I8" s="10"/>
+      <c r="I8" s="9"/>
       <c r="J8" s="9"/>
       <c r="K8" s="9"/>
-      <c r="L8" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
+      <c r="L8" s="11">
+        <v>6</v>
+      </c>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
       <c r="O8" s="9"/>
       <c r="P8" s="9"/>
-      <c r="Q8" s="4"/>
-      <c r="R8" s="11" t="s">
+      <c r="Q8" s="10"/>
+      <c r="R8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="S8" s="4"/>
-      <c r="T8" s="4" t="s">
+      <c r="S8" s="10"/>
+      <c r="T8" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="U8" s="4"/>
-      <c r="V8" s="4"/>
-      <c r="W8" s="4"/>
-      <c r="X8" s="4"/>
-      <c r="Y8" s="4"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="3"/>
+      <c r="W8" s="3"/>
+      <c r="X8" s="3"/>
+      <c r="Y8" s="3"/>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B9" s="9"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9"/>
-      <c r="I9" s="10"/>
+      <c r="I9" s="9"/>
       <c r="J9" s="9"/>
       <c r="K9" s="9"/>
-      <c r="L9" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
+      <c r="L9" s="11">
+        <v>2</v>
+      </c>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
       <c r="O9" s="9"/>
       <c r="P9" s="9"/>
-      <c r="Q9" s="8"/>
-      <c r="R9" s="4"/>
-      <c r="S9" s="4"/>
-      <c r="T9" s="4"/>
-      <c r="U9" s="4"/>
-      <c r="V9" s="4"/>
-      <c r="W9" s="4"/>
-      <c r="X9" s="4"/>
-      <c r="Y9" s="4"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="10"/>
+      <c r="S9" s="10"/>
+      <c r="T9" s="10"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="3"/>
+      <c r="X9" s="3"/>
+      <c r="Y9" s="3"/>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="9"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9"/>
-      <c r="I10" s="10"/>
+      <c r="I10" s="9"/>
       <c r="J10" s="9"/>
       <c r="K10" s="9"/>
-      <c r="L10" s="12">
+      <c r="L10" s="11">
         <v>3</v>
       </c>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
       <c r="O10" s="9"/>
       <c r="P10" s="9"/>
-      <c r="Q10" s="4"/>
-      <c r="R10" s="4"/>
-      <c r="S10" s="4"/>
-      <c r="T10" s="4"/>
-      <c r="U10" s="4"/>
-      <c r="V10" s="4"/>
-      <c r="W10" s="4"/>
-      <c r="X10" s="4"/>
-      <c r="Y10" s="4"/>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="10"/>
+      <c r="S10" s="10"/>
+      <c r="T10" s="10"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3"/>
+      <c r="X10" s="3"/>
+      <c r="Y10" s="3"/>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="9"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
       <c r="F11" s="9"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
-      <c r="I11" s="10"/>
+      <c r="I11" s="9"/>
       <c r="J11" s="9"/>
       <c r="K11" s="9"/>
-      <c r="L11" s="12">
+      <c r="L11" s="11">
         <v>3</v>
       </c>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
       <c r="O11" s="9"/>
       <c r="P11" s="9"/>
-      <c r="Q11" s="4"/>
-      <c r="R11" s="4"/>
-      <c r="S11" s="4"/>
-      <c r="T11" s="4"/>
-      <c r="U11" s="4"/>
-      <c r="V11" s="4"/>
-      <c r="W11" s="4"/>
-      <c r="X11" s="4"/>
-      <c r="Y11" s="4"/>
+      <c r="Q11" s="10"/>
+      <c r="R11" s="10"/>
+      <c r="S11" s="10"/>
+      <c r="T11" s="10"/>
+      <c r="U11" s="10"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="3"/>
+      <c r="X11" s="3"/>
+      <c r="Y11" s="3"/>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B12" s="9"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
       <c r="F12" s="9"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
-      <c r="I12" s="10"/>
+      <c r="I12" s="9"/>
       <c r="J12" s="9"/>
       <c r="K12" s="9"/>
-      <c r="L12" s="12">
+      <c r="L12" s="11">
         <v>4</v>
       </c>
-      <c r="M12" s="10"/>
-      <c r="N12" s="10"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
       <c r="O12" s="9"/>
       <c r="P12" s="9"/>
-      <c r="Q12" s="4"/>
-      <c r="R12" s="4"/>
-      <c r="S12" s="4"/>
-      <c r="T12" s="4"/>
-      <c r="U12" s="4"/>
-      <c r="V12" s="4"/>
-      <c r="W12" s="4"/>
-      <c r="X12" s="4"/>
-      <c r="Y12" s="4"/>
+      <c r="Q12" s="10"/>
+      <c r="R12" s="10"/>
+      <c r="S12" s="10"/>
+      <c r="T12" s="10"/>
+      <c r="U12" s="10"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="3"/>
+      <c r="X12" s="3"/>
+      <c r="Y12" s="3"/>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="9"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
-      <c r="I13" s="10"/>
+      <c r="I13" s="9"/>
       <c r="J13" s="9"/>
       <c r="K13" s="9"/>
-      <c r="L13" s="12">
+      <c r="L13" s="11">
         <v>4</v>
       </c>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
       <c r="O13" s="9"/>
       <c r="P13" s="9"/>
-      <c r="Q13" s="4"/>
-      <c r="R13" s="4"/>
-      <c r="S13" s="4"/>
-      <c r="T13" s="4"/>
-      <c r="U13" s="4"/>
-      <c r="V13" s="4"/>
-      <c r="W13" s="4"/>
-      <c r="X13" s="4"/>
-      <c r="Y13" s="4"/>
+      <c r="Q13" s="10"/>
+      <c r="R13" s="10"/>
+      <c r="S13" s="10"/>
+      <c r="T13" s="10"/>
+      <c r="U13" s="10"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
+      <c r="X13" s="3"/>
+      <c r="Y13" s="3"/>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B14" s="9"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
       <c r="F14" s="9"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
-      <c r="I14" s="10"/>
+      <c r="I14" s="9"/>
       <c r="J14" s="9"/>
       <c r="K14" s="9"/>
-      <c r="L14" s="12">
+      <c r="L14" s="11">
         <v>4</v>
       </c>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
       <c r="O14" s="9"/>
       <c r="P14" s="9"/>
-      <c r="Q14" s="4"/>
-      <c r="R14" s="4"/>
-      <c r="S14" s="4"/>
-      <c r="T14" s="4"/>
-      <c r="U14" s="4"/>
-      <c r="V14" s="4"/>
-      <c r="W14" s="4"/>
-      <c r="X14" s="4"/>
-      <c r="Y14" s="4"/>
+      <c r="Q14" s="10"/>
+      <c r="R14" s="10"/>
+      <c r="S14" s="10"/>
+      <c r="T14" s="10"/>
+      <c r="U14" s="10"/>
+      <c r="V14" s="3"/>
+      <c r="W14" s="3"/>
+      <c r="X14" s="3"/>
+      <c r="Y14" s="3"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B15" s="9"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
       <c r="F15" s="9"/>
       <c r="G15" s="9"/>
       <c r="H15" s="9"/>
-      <c r="I15" s="10"/>
+      <c r="I15" s="9"/>
       <c r="J15" s="9"/>
       <c r="K15" s="9"/>
-      <c r="L15" s="12">
+      <c r="L15" s="11">
         <v>5</v>
       </c>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
       <c r="O15" s="9"/>
       <c r="P15" s="9"/>
-      <c r="Q15" s="4"/>
-      <c r="R15" s="4"/>
-      <c r="S15" s="4"/>
-      <c r="T15" s="4"/>
-      <c r="U15" s="4"/>
-      <c r="V15" s="4"/>
-      <c r="W15" s="4"/>
-      <c r="X15" s="4"/>
-      <c r="Y15" s="4"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="10"/>
+      <c r="U15" s="10"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="3"/>
+      <c r="X15" s="3"/>
+      <c r="Y15" s="3"/>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="9"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
       <c r="F16" s="9"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
-      <c r="I16" s="10"/>
+      <c r="I16" s="9"/>
       <c r="J16" s="9"/>
       <c r="K16" s="9"/>
-      <c r="L16" s="12">
+      <c r="L16" s="11">
         <v>5</v>
       </c>
-      <c r="M16" s="10"/>
-      <c r="N16" s="10"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
       <c r="O16" s="9"/>
       <c r="P16" s="9"/>
-      <c r="Q16" s="4"/>
-      <c r="R16" s="4"/>
-      <c r="S16" s="4"/>
-      <c r="T16" s="4"/>
-      <c r="U16" s="4"/>
-      <c r="V16" s="4"/>
-      <c r="W16" s="4"/>
-      <c r="X16" s="4"/>
-      <c r="Y16" s="4"/>
+      <c r="Q16" s="10"/>
+      <c r="R16" s="10"/>
+      <c r="S16" s="10"/>
+      <c r="T16" s="10"/>
+      <c r="U16" s="10"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="3"/>
+      <c r="X16" s="3"/>
+      <c r="Y16" s="3"/>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="9"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
       <c r="F17" s="9"/>
       <c r="G17" s="9"/>
       <c r="H17" s="9"/>
-      <c r="I17" s="10"/>
+      <c r="I17" s="9"/>
       <c r="J17" s="9"/>
       <c r="K17" s="9"/>
-      <c r="L17" s="12">
+      <c r="L17" s="11">
         <v>6</v>
       </c>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
       <c r="O17" s="9"/>
       <c r="P17" s="9"/>
-      <c r="Q17" s="4"/>
-      <c r="R17" s="4"/>
-      <c r="S17" s="4"/>
-      <c r="T17" s="4"/>
-      <c r="U17" s="4"/>
-      <c r="V17" s="4"/>
-      <c r="W17" s="4"/>
-      <c r="X17" s="4"/>
-      <c r="Y17" s="4"/>
+      <c r="Q17" s="10"/>
+      <c r="R17" s="10"/>
+      <c r="S17" s="10"/>
+      <c r="T17" s="10"/>
+      <c r="U17" s="10"/>
+      <c r="V17" s="3"/>
+      <c r="W17" s="3"/>
+      <c r="X17" s="3"/>
+      <c r="Y17" s="3"/>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B18" s="9"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
       <c r="H18" s="9"/>
-      <c r="I18" s="10"/>
+      <c r="I18" s="9"/>
       <c r="J18" s="9"/>
       <c r="K18" s="9"/>
-      <c r="L18" s="13">
+      <c r="L18" s="8">
         <v>6</v>
       </c>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
       <c r="O18" s="9"/>
       <c r="P18" s="9"/>
-      <c r="Q18" s="4"/>
-      <c r="R18" s="4"/>
-      <c r="S18" s="4"/>
-      <c r="T18" s="4"/>
-      <c r="U18" s="4"/>
-      <c r="V18" s="4"/>
-      <c r="W18" s="4"/>
-      <c r="X18" s="4"/>
-      <c r="Y18" s="4"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+      <c r="S18" s="10"/>
+      <c r="T18" s="10"/>
+      <c r="U18" s="10"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="3"/>
+      <c r="X18" s="3"/>
+      <c r="Y18" s="3"/>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A19" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="9"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
       <c r="H19" s="9"/>
-      <c r="I19" s="10"/>
+      <c r="I19" s="9"/>
       <c r="J19" s="9"/>
       <c r="K19" s="9"/>
-      <c r="L19" s="14">
+      <c r="L19" s="8">
         <v>3</v>
       </c>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10"/>
+      <c r="M19" s="9"/>
+      <c r="N19" s="9"/>
       <c r="O19" s="9"/>
       <c r="P19" s="9"/>
-      <c r="Q19" s="4"/>
-      <c r="R19" s="4"/>
-      <c r="S19" s="4"/>
-      <c r="T19" s="4"/>
-      <c r="U19" s="4"/>
-      <c r="V19" s="4"/>
-      <c r="W19" s="4"/>
-      <c r="X19" s="4"/>
-      <c r="Y19" s="4"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="10"/>
+      <c r="U19" s="10"/>
+      <c r="V19" s="3"/>
+      <c r="W19" s="3"/>
+      <c r="X19" s="3"/>
+      <c r="Y19" s="3"/>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B20" s="9"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
       <c r="H20" s="9"/>
-      <c r="I20" s="10"/>
+      <c r="I20" s="9"/>
       <c r="J20" s="9"/>
       <c r="K20" s="9"/>
-      <c r="L20" s="12">
+      <c r="L20" s="11">
         <v>4</v>
       </c>
-      <c r="M20" s="10"/>
-      <c r="N20" s="10"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
       <c r="O20" s="9"/>
       <c r="P20" s="9"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="10"/>
+      <c r="S20" s="10"/>
+      <c r="T20" s="10"/>
+      <c r="U20" s="10"/>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B21" s="9"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
       <c r="H21" s="9"/>
-      <c r="I21" s="10"/>
+      <c r="I21" s="9"/>
       <c r="J21" s="9"/>
       <c r="K21" s="9"/>
-      <c r="L21" s="12">
+      <c r="L21" s="11">
         <v>4</v>
       </c>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
       <c r="O21" s="9"/>
       <c r="P21" s="9"/>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="10"/>
+      <c r="S21" s="10"/>
+      <c r="T21" s="10"/>
+      <c r="U21" s="10"/>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A22" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="9"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
       <c r="H22" s="9"/>
-      <c r="I22" s="10"/>
+      <c r="I22" s="9"/>
       <c r="J22" s="9"/>
       <c r="K22" s="9"/>
-      <c r="L22" s="12">
+      <c r="L22" s="11">
         <v>4</v>
       </c>
-      <c r="M22" s="10"/>
-      <c r="N22" s="10"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
       <c r="O22" s="9"/>
       <c r="P22" s="9"/>
+      <c r="Q22" s="10"/>
+      <c r="R22" s="10"/>
+      <c r="S22" s="10"/>
+      <c r="T22" s="10"/>
+      <c r="U22" s="10"/>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A23" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B23" s="9"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
-      <c r="I23" s="10"/>
+      <c r="I23" s="9"/>
       <c r="J23" s="9"/>
       <c r="K23" s="9"/>
-      <c r="L23" s="12">
+      <c r="L23" s="11">
         <v>5</v>
       </c>
-      <c r="M23" s="10"/>
-      <c r="N23" s="10"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="9"/>
       <c r="O23" s="9"/>
       <c r="P23" s="9"/>
+      <c r="Q23" s="10"/>
+      <c r="R23" s="10"/>
+      <c r="S23" s="10"/>
+      <c r="T23" s="10"/>
+      <c r="U23" s="10"/>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A24" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B24" s="9"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
       <c r="H24" s="9"/>
-      <c r="I24" s="10"/>
+      <c r="I24" s="9"/>
       <c r="J24" s="9"/>
       <c r="K24" s="9"/>
-      <c r="L24" s="12">
+      <c r="L24" s="11">
         <v>5</v>
       </c>
-      <c r="M24" s="10"/>
-      <c r="N24" s="10"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="9"/>
       <c r="O24" s="9"/>
       <c r="P24" s="9"/>
+      <c r="Q24" s="10"/>
+      <c r="R24" s="10"/>
+      <c r="S24" s="10"/>
+      <c r="T24" s="10"/>
+      <c r="U24" s="10"/>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A25" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B25" s="9"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
-      <c r="I25" s="10"/>
+      <c r="I25" s="9"/>
       <c r="J25" s="9"/>
       <c r="K25" s="9"/>
-      <c r="L25" s="12">
+      <c r="L25" s="11">
         <v>5</v>
       </c>
-      <c r="M25" s="10"/>
-      <c r="N25" s="10"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
       <c r="O25" s="9"/>
       <c r="P25" s="9"/>
       <c r="Q25" s="6"/>
+      <c r="R25" s="10"/>
+      <c r="S25" s="10"/>
+      <c r="T25" s="10"/>
+      <c r="U25" s="10"/>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A26" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B26" s="9"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
-      <c r="I26" s="10"/>
+      <c r="I26" s="9"/>
       <c r="J26" s="9"/>
       <c r="K26" s="9"/>
-      <c r="L26" s="12">
+      <c r="L26" s="11">
         <v>6</v>
       </c>
-      <c r="M26" s="10"/>
-      <c r="N26" s="10"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9"/>
       <c r="O26" s="9"/>
       <c r="P26" s="9"/>
+      <c r="Q26" s="10"/>
+      <c r="R26" s="10"/>
+      <c r="S26" s="10"/>
+      <c r="T26" s="10"/>
+      <c r="U26" s="10"/>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B27" s="9"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
       <c r="H27" s="9"/>
-      <c r="I27" s="10"/>
+      <c r="I27" s="9"/>
       <c r="J27" s="9"/>
       <c r="K27" s="9"/>
-      <c r="L27" s="2">
+      <c r="L27" s="11">
         <v>6</v>
       </c>
-      <c r="M27" s="10"/>
-      <c r="N27" s="10"/>
+      <c r="M27" s="9"/>
+      <c r="N27" s="9"/>
       <c r="O27" s="9"/>
       <c r="P27" s="9"/>
+      <c r="Q27" s="10"/>
+      <c r="R27" s="10"/>
+      <c r="S27" s="10"/>
+      <c r="T27" s="10"/>
+      <c r="U27" s="10"/>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A28" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B28" s="9"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
       <c r="H28" s="9"/>
-      <c r="I28" s="10"/>
+      <c r="I28" s="9"/>
       <c r="J28" s="9"/>
       <c r="K28" s="9"/>
-      <c r="L28" s="2">
+      <c r="L28" s="11">
         <v>6</v>
       </c>
-      <c r="M28" s="10"/>
-      <c r="N28" s="10"/>
+      <c r="M28" s="9"/>
+      <c r="N28" s="9"/>
       <c r="O28" s="9"/>
       <c r="P28" s="9"/>
+      <c r="Q28" s="10"/>
+      <c r="R28" s="10"/>
+      <c r="S28" s="10"/>
+      <c r="T28" s="10"/>
+      <c r="U28" s="10"/>
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A29" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B29" s="9"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
       <c r="H29" s="9"/>
-      <c r="I29" s="10"/>
+      <c r="I29" s="9"/>
       <c r="J29" s="9"/>
       <c r="K29" s="9"/>
-      <c r="L29" s="2">
+      <c r="L29" s="11">
         <v>4</v>
       </c>
-      <c r="M29" s="10"/>
-      <c r="N29" s="10"/>
+      <c r="M29" s="9"/>
+      <c r="N29" s="9"/>
       <c r="O29" s="9"/>
       <c r="P29" s="9"/>
+      <c r="Q29" s="10"/>
+      <c r="R29" s="10"/>
+      <c r="S29" s="10"/>
+      <c r="T29" s="10"/>
+      <c r="U29" s="10"/>
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A30" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B30" s="9"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
       <c r="H30" s="9"/>
-      <c r="I30" s="10"/>
+      <c r="I30" s="9"/>
       <c r="J30" s="9"/>
       <c r="K30" s="9"/>
-      <c r="L30" s="2">
+      <c r="L30" s="11">
         <v>5</v>
       </c>
-      <c r="M30" s="10"/>
-      <c r="N30" s="10"/>
+      <c r="M30" s="9"/>
+      <c r="N30" s="9"/>
       <c r="O30" s="9"/>
       <c r="P30" s="9"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="10"/>
+      <c r="S30" s="10"/>
+      <c r="T30" s="10"/>
+      <c r="U30" s="10"/>
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A31" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B31" s="9"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
-      <c r="I31" s="10"/>
+      <c r="I31" s="9"/>
       <c r="J31" s="9"/>
       <c r="K31" s="9"/>
-      <c r="L31" s="2">
+      <c r="L31" s="11">
         <v>5</v>
       </c>
-      <c r="M31" s="10"/>
-      <c r="N31" s="10"/>
+      <c r="M31" s="9"/>
+      <c r="N31" s="9"/>
       <c r="O31" s="9"/>
       <c r="P31" s="9"/>
+      <c r="Q31" s="10"/>
+      <c r="R31" s="10"/>
+      <c r="S31" s="10"/>
+      <c r="T31" s="10"/>
+      <c r="U31" s="10"/>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A32" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B32" s="9"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
-      <c r="I32" s="10"/>
+      <c r="I32" s="9"/>
       <c r="J32" s="9"/>
       <c r="K32" s="9"/>
-      <c r="L32" s="2">
+      <c r="L32" s="11">
         <v>5</v>
       </c>
-      <c r="M32" s="10"/>
-      <c r="N32" s="10"/>
+      <c r="M32" s="9"/>
+      <c r="N32" s="9"/>
       <c r="O32" s="9"/>
       <c r="P32" s="9"/>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q32" s="10"/>
+      <c r="R32" s="10"/>
+      <c r="S32" s="10"/>
+      <c r="T32" s="10"/>
+      <c r="U32" s="10"/>
+    </row>
+    <row r="33" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A33" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B33" s="9"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
-      <c r="I33" s="10"/>
+      <c r="I33" s="9"/>
       <c r="J33" s="9"/>
       <c r="K33" s="9"/>
-      <c r="L33" s="2">
+      <c r="L33" s="11">
         <v>5</v>
       </c>
-      <c r="M33" s="10"/>
-      <c r="N33" s="10"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
       <c r="O33" s="9"/>
       <c r="P33" s="9"/>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q33" s="10"/>
+      <c r="R33" s="10"/>
+      <c r="S33" s="10"/>
+      <c r="T33" s="10"/>
+      <c r="U33" s="10"/>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A34" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B34" s="9"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
       <c r="H34" s="9"/>
-      <c r="I34" s="10"/>
+      <c r="I34" s="9"/>
       <c r="J34" s="9"/>
       <c r="K34" s="9"/>
-      <c r="L34" s="2">
+      <c r="L34" s="11">
         <v>5</v>
       </c>
-      <c r="M34" s="10"/>
-      <c r="N34" s="10"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
       <c r="O34" s="9"/>
       <c r="P34" s="9"/>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q34" s="10"/>
+      <c r="R34" s="10"/>
+      <c r="S34" s="10"/>
+      <c r="T34" s="10"/>
+      <c r="U34" s="10"/>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A35" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B35" s="9"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
       <c r="H35" s="9"/>
-      <c r="I35" s="10"/>
+      <c r="I35" s="9"/>
       <c r="J35" s="9"/>
       <c r="K35" s="9"/>
-      <c r="L35" s="2">
+      <c r="L35" s="11">
         <v>5</v>
       </c>
-      <c r="M35" s="10"/>
-      <c r="N35" s="10"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
       <c r="O35" s="9"/>
       <c r="P35" s="9"/>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q35" s="10"/>
+      <c r="R35" s="10"/>
+      <c r="S35" s="10"/>
+      <c r="T35" s="10"/>
+      <c r="U35" s="10"/>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A36" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B36" s="9"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
       <c r="H36" s="9"/>
-      <c r="I36" s="10"/>
+      <c r="I36" s="9"/>
       <c r="J36" s="9"/>
       <c r="K36" s="9"/>
-      <c r="L36" s="2">
+      <c r="L36" s="11">
         <v>5</v>
       </c>
-      <c r="M36" s="10"/>
-      <c r="N36" s="10"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
       <c r="O36" s="9"/>
       <c r="P36" s="9"/>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q36" s="10"/>
+      <c r="R36" s="10"/>
+      <c r="S36" s="10"/>
+      <c r="T36" s="10"/>
+      <c r="U36" s="10"/>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A37" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B37" s="9"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
       <c r="H37" s="9"/>
-      <c r="I37" s="10"/>
+      <c r="I37" s="9"/>
       <c r="J37" s="9"/>
       <c r="K37" s="9"/>
-      <c r="L37" s="2">
+      <c r="L37" s="11">
         <v>5</v>
       </c>
-      <c r="M37" s="10"/>
-      <c r="N37" s="10"/>
+      <c r="M37" s="9"/>
+      <c r="N37" s="9"/>
       <c r="O37" s="9"/>
       <c r="P37" s="9"/>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q37" s="10"/>
+      <c r="R37" s="10"/>
+      <c r="S37" s="10"/>
+      <c r="T37" s="10"/>
+      <c r="U37" s="10"/>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A38" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B38" s="9"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
       <c r="H38" s="9"/>
-      <c r="I38" s="10"/>
+      <c r="I38" s="9"/>
       <c r="J38" s="9"/>
       <c r="K38" s="9"/>
-      <c r="L38" s="2">
+      <c r="L38" s="11">
         <v>6</v>
       </c>
-      <c r="M38" s="10"/>
-      <c r="N38" s="10"/>
+      <c r="M38" s="9"/>
+      <c r="N38" s="9"/>
       <c r="O38" s="9"/>
       <c r="P38" s="9"/>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q38" s="10"/>
+      <c r="R38" s="10"/>
+      <c r="S38" s="10"/>
+      <c r="T38" s="10"/>
+      <c r="U38" s="10"/>
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A39" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B39" s="9"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
       <c r="H39" s="9"/>
-      <c r="I39" s="10"/>
+      <c r="I39" s="9"/>
       <c r="J39" s="9"/>
       <c r="K39" s="9"/>
-      <c r="L39" s="2">
+      <c r="L39" s="11">
         <v>6</v>
       </c>
-      <c r="M39" s="10"/>
-      <c r="N39" s="10"/>
+      <c r="M39" s="9"/>
+      <c r="N39" s="9"/>
       <c r="O39" s="9"/>
       <c r="P39" s="9"/>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q39" s="10"/>
+      <c r="R39" s="10"/>
+      <c r="S39" s="10"/>
+      <c r="T39" s="10"/>
+      <c r="U39" s="10"/>
+    </row>
+    <row r="40" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A40" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B40" s="9"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
       <c r="H40" s="9"/>
-      <c r="I40" s="10"/>
+      <c r="I40" s="9"/>
       <c r="J40" s="9"/>
       <c r="K40" s="9"/>
-      <c r="L40" s="2">
+      <c r="L40" s="11">
         <v>6</v>
       </c>
-      <c r="M40" s="10"/>
-      <c r="N40" s="10"/>
+      <c r="M40" s="9"/>
+      <c r="N40" s="9"/>
       <c r="O40" s="9"/>
       <c r="P40" s="9"/>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q40" s="10"/>
+      <c r="R40" s="10"/>
+      <c r="S40" s="10"/>
+      <c r="T40" s="10"/>
+      <c r="U40" s="10"/>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A41" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B41" s="9"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
-      <c r="E41" s="10"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
       <c r="F41" s="9"/>
       <c r="G41" s="9"/>
       <c r="H41" s="9"/>
-      <c r="I41" s="10"/>
+      <c r="I41" s="9"/>
       <c r="J41" s="9"/>
       <c r="K41" s="9"/>
-      <c r="L41" s="2">
+      <c r="L41" s="11">
         <v>6</v>
       </c>
-      <c r="M41" s="10"/>
-      <c r="N41" s="10"/>
+      <c r="M41" s="9"/>
+      <c r="N41" s="9"/>
       <c r="O41" s="9"/>
       <c r="P41" s="9"/>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q41" s="10"/>
+      <c r="R41" s="10"/>
+      <c r="S41" s="10"/>
+      <c r="T41" s="10"/>
+      <c r="U41" s="10"/>
+    </row>
+    <row r="42" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A42" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B42" s="9"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
       <c r="F42" s="9"/>
       <c r="G42" s="9"/>
       <c r="H42" s="9"/>
-      <c r="I42" s="10"/>
+      <c r="I42" s="9"/>
       <c r="J42" s="9"/>
       <c r="K42" s="9"/>
-      <c r="L42" s="2">
+      <c r="L42" s="11">
         <v>6</v>
       </c>
-      <c r="M42" s="10"/>
-      <c r="N42" s="10"/>
+      <c r="M42" s="9"/>
+      <c r="N42" s="9"/>
       <c r="O42" s="9"/>
       <c r="P42" s="9"/>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q42" s="10"/>
+      <c r="R42" s="10"/>
+      <c r="S42" s="10"/>
+      <c r="T42" s="10"/>
+      <c r="U42" s="10"/>
+    </row>
+    <row r="43" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A43" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B43" s="9"/>
-      <c r="C43" s="10"/>
-      <c r="D43" s="10"/>
-      <c r="E43" s="10"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
       <c r="H43" s="9"/>
-      <c r="I43" s="10"/>
+      <c r="I43" s="9"/>
       <c r="J43" s="9"/>
       <c r="K43" s="9"/>
-      <c r="L43" s="2">
+      <c r="L43" s="11">
         <v>6</v>
       </c>
-      <c r="M43" s="10"/>
-      <c r="N43" s="10"/>
+      <c r="M43" s="9"/>
+      <c r="N43" s="9"/>
       <c r="O43" s="9"/>
       <c r="P43" s="9"/>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q43" s="10"/>
+      <c r="R43" s="10"/>
+      <c r="S43" s="10"/>
+      <c r="T43" s="10"/>
+      <c r="U43" s="10"/>
+    </row>
+    <row r="44" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A44" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B44" s="9"/>
-      <c r="C44" s="10"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="10"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
       <c r="H44" s="9"/>
-      <c r="I44" s="10"/>
+      <c r="I44" s="9"/>
       <c r="J44" s="9"/>
       <c r="K44" s="9"/>
-      <c r="L44" s="2">
+      <c r="L44" s="11">
         <v>6</v>
       </c>
-      <c r="M44" s="10"/>
-      <c r="N44" s="10"/>
+      <c r="M44" s="9"/>
+      <c r="N44" s="9"/>
       <c r="O44" s="9"/>
       <c r="P44" s="9"/>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q44" s="10"/>
+      <c r="R44" s="10"/>
+      <c r="S44" s="10"/>
+      <c r="T44" s="10"/>
+      <c r="U44" s="10"/>
+    </row>
+    <row r="45" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A45" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B45" s="9"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="10"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
       <c r="F45" s="9"/>
       <c r="G45" s="9"/>
       <c r="H45" s="9"/>
-      <c r="I45" s="10"/>
+      <c r="I45" s="9"/>
       <c r="J45" s="9"/>
       <c r="K45" s="9"/>
-      <c r="L45" s="2">
+      <c r="L45" s="11">
         <v>4</v>
       </c>
-      <c r="M45" s="10"/>
-      <c r="N45" s="10"/>
+      <c r="M45" s="9"/>
+      <c r="N45" s="9"/>
       <c r="O45" s="9"/>
       <c r="P45" s="9"/>
-    </row>
-    <row r="46" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="Q45" s="10"/>
+      <c r="R45" s="10"/>
+      <c r="S45" s="10"/>
+      <c r="T45" s="10"/>
+      <c r="U45" s="10"/>
+    </row>
+    <row r="46" spans="1:21" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B46" s="9"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
       <c r="H46" s="9"/>
-      <c r="I46" s="10"/>
+      <c r="I46" s="9"/>
       <c r="J46" s="9"/>
       <c r="K46" s="9"/>
-      <c r="L46" s="2">
+      <c r="L46" s="11">
         <v>5</v>
       </c>
-      <c r="M46" s="10"/>
-      <c r="N46" s="10"/>
+      <c r="M46" s="9"/>
+      <c r="N46" s="9"/>
       <c r="O46" s="9"/>
       <c r="P46" s="9"/>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q46" s="10"/>
+      <c r="R46" s="10"/>
+      <c r="S46" s="10"/>
+      <c r="T46" s="10"/>
+      <c r="U46" s="10"/>
+    </row>
+    <row r="47" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A47" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B47" s="9"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
       <c r="H47" s="9"/>
-      <c r="I47" s="10"/>
+      <c r="I47" s="9"/>
       <c r="J47" s="9"/>
       <c r="K47" s="9"/>
-      <c r="L47" s="2">
+      <c r="L47" s="11">
         <v>5</v>
       </c>
-      <c r="M47" s="10"/>
-      <c r="N47" s="10"/>
+      <c r="M47" s="9"/>
+      <c r="N47" s="9"/>
       <c r="O47" s="9"/>
       <c r="P47" s="9"/>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q47" s="10"/>
+      <c r="R47" s="10"/>
+      <c r="S47" s="10"/>
+      <c r="T47" s="10"/>
+      <c r="U47" s="10"/>
+    </row>
+    <row r="48" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A48" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B48" s="9"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
       <c r="H48" s="9"/>
-      <c r="I48" s="10"/>
+      <c r="I48" s="9"/>
       <c r="J48" s="9"/>
       <c r="K48" s="9"/>
-      <c r="L48" s="2">
+      <c r="L48" s="11">
         <v>5</v>
       </c>
-      <c r="M48" s="10"/>
-      <c r="N48" s="10"/>
+      <c r="M48" s="9"/>
+      <c r="N48" s="9"/>
       <c r="O48" s="9"/>
       <c r="P48" s="9"/>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q48" s="10"/>
+      <c r="R48" s="10"/>
+      <c r="S48" s="10"/>
+      <c r="T48" s="10"/>
+      <c r="U48" s="10"/>
+    </row>
+    <row r="49" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B49" s="9"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="10"/>
-      <c r="E49" s="10"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
       <c r="H49" s="9"/>
-      <c r="I49" s="10"/>
+      <c r="I49" s="9"/>
       <c r="J49" s="9"/>
       <c r="K49" s="9"/>
-      <c r="L49" s="2">
+      <c r="L49" s="11">
         <v>5</v>
       </c>
-      <c r="M49" s="10"/>
-      <c r="N49" s="10"/>
+      <c r="M49" s="9"/>
+      <c r="N49" s="9"/>
       <c r="O49" s="9"/>
       <c r="P49" s="9"/>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q49" s="10"/>
+      <c r="R49" s="10"/>
+      <c r="S49" s="10"/>
+      <c r="T49" s="10"/>
+      <c r="U49" s="10"/>
+    </row>
+    <row r="50" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B50" s="9"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
+      <c r="C50" s="9"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="9"/>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
       <c r="H50" s="9"/>
-      <c r="I50" s="10"/>
+      <c r="I50" s="9"/>
       <c r="J50" s="9"/>
       <c r="K50" s="9"/>
-      <c r="L50" s="2">
+      <c r="L50" s="11">
         <v>6</v>
       </c>
-      <c r="M50" s="10"/>
-      <c r="N50" s="10"/>
+      <c r="M50" s="9"/>
+      <c r="N50" s="9"/>
       <c r="O50" s="9"/>
       <c r="P50" s="9"/>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q50" s="10"/>
+      <c r="R50" s="10"/>
+      <c r="S50" s="10"/>
+      <c r="T50" s="10"/>
+      <c r="U50" s="10"/>
+    </row>
+    <row r="51" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B51" s="9"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
       <c r="F51" s="9"/>
       <c r="G51" s="9"/>
       <c r="H51" s="9"/>
-      <c r="I51" s="10"/>
+      <c r="I51" s="9"/>
       <c r="J51" s="9"/>
       <c r="K51" s="9"/>
-      <c r="L51" s="2">
+      <c r="L51" s="11">
         <v>6</v>
       </c>
-      <c r="M51" s="10"/>
-      <c r="N51" s="10"/>
+      <c r="M51" s="9"/>
+      <c r="N51" s="9"/>
       <c r="O51" s="9"/>
       <c r="P51" s="9"/>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q51" s="10"/>
+      <c r="R51" s="10"/>
+      <c r="S51" s="10"/>
+      <c r="T51" s="10"/>
+      <c r="U51" s="10"/>
+    </row>
+    <row r="52" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B52" s="9"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="10"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
       <c r="F52" s="9"/>
       <c r="G52" s="9"/>
       <c r="H52" s="9"/>
-      <c r="I52" s="10"/>
+      <c r="I52" s="9"/>
       <c r="J52" s="9"/>
       <c r="K52" s="9"/>
-      <c r="L52" s="2">
+      <c r="L52" s="11">
         <v>6</v>
       </c>
-      <c r="M52" s="10"/>
-      <c r="N52" s="10"/>
+      <c r="M52" s="9"/>
+      <c r="N52" s="9"/>
       <c r="O52" s="9"/>
       <c r="P52" s="9"/>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q52" s="10"/>
+      <c r="R52" s="10"/>
+      <c r="S52" s="10"/>
+      <c r="T52" s="10"/>
+      <c r="U52" s="10"/>
+    </row>
+    <row r="53" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A53" s="9" t="s">
         <v>23</v>
       </c>
       <c r="B53" s="9"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="10"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
       <c r="H53" s="9"/>
-      <c r="I53" s="10"/>
+      <c r="I53" s="9"/>
       <c r="J53" s="9"/>
       <c r="K53" s="9"/>
-      <c r="L53" s="2">
+      <c r="L53" s="11">
         <v>5</v>
       </c>
-      <c r="M53" s="10"/>
-      <c r="N53" s="10"/>
+      <c r="M53" s="9"/>
+      <c r="N53" s="9"/>
       <c r="O53" s="9"/>
       <c r="P53" s="9"/>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q53" s="10"/>
+      <c r="R53" s="10"/>
+      <c r="S53" s="10"/>
+      <c r="T53" s="10"/>
+      <c r="U53" s="10"/>
+    </row>
+    <row r="54" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A54" s="9" t="s">
         <v>23</v>
       </c>
       <c r="B54" s="9"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="10"/>
-      <c r="E54" s="10"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
       <c r="H54" s="9"/>
-      <c r="I54" s="10"/>
+      <c r="I54" s="9"/>
       <c r="J54" s="9"/>
       <c r="K54" s="9"/>
-      <c r="L54" s="2">
+      <c r="L54" s="11">
         <v>6</v>
       </c>
-      <c r="M54" s="10"/>
-      <c r="N54" s="10"/>
+      <c r="M54" s="9"/>
+      <c r="N54" s="9"/>
       <c r="O54" s="9"/>
       <c r="P54" s="9"/>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q54" s="10"/>
+      <c r="R54" s="10"/>
+      <c r="S54" s="10"/>
+      <c r="T54" s="10"/>
+      <c r="U54" s="10"/>
+    </row>
+    <row r="55" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A55" s="9" t="s">
         <v>23</v>
       </c>
       <c r="B55" s="9"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="10"/>
-      <c r="E55" s="10"/>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
       <c r="H55" s="9"/>
-      <c r="I55" s="10"/>
+      <c r="I55" s="9"/>
       <c r="J55" s="9"/>
       <c r="K55" s="9"/>
-      <c r="L55" s="2">
+      <c r="L55" s="11">
         <v>6</v>
       </c>
-      <c r="M55" s="10"/>
-      <c r="N55" s="10"/>
+      <c r="M55" s="9"/>
+      <c r="N55" s="9"/>
       <c r="O55" s="9"/>
       <c r="P55" s="9"/>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q55" s="10"/>
+      <c r="R55" s="10"/>
+      <c r="S55" s="10"/>
+      <c r="T55" s="10"/>
+      <c r="U55" s="10"/>
+    </row>
+    <row r="56" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A56" s="9" t="s">
         <v>23</v>
       </c>
       <c r="B56" s="9"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
       <c r="F56" s="9"/>
       <c r="G56" s="9"/>
       <c r="H56" s="9"/>
-      <c r="I56" s="10"/>
+      <c r="I56" s="9"/>
       <c r="J56" s="9"/>
       <c r="K56" s="9"/>
-      <c r="L56" s="2">
+      <c r="L56" s="11">
         <v>6</v>
       </c>
-      <c r="M56" s="10"/>
-      <c r="N56" s="10"/>
+      <c r="M56" s="9"/>
+      <c r="N56" s="9"/>
       <c r="O56" s="9"/>
       <c r="P56" s="9"/>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q56" s="10"/>
+      <c r="R56" s="10"/>
+      <c r="S56" s="10"/>
+      <c r="T56" s="10"/>
+      <c r="U56" s="10"/>
+    </row>
+    <row r="57" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A57" s="9" t="s">
         <v>23</v>
       </c>
       <c r="B57" s="9"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="10"/>
-      <c r="E57" s="10"/>
+      <c r="C57" s="9"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="9"/>
       <c r="F57" s="9"/>
       <c r="G57" s="9"/>
       <c r="H57" s="9"/>
-      <c r="I57" s="10"/>
+      <c r="I57" s="9"/>
       <c r="J57" s="9"/>
       <c r="K57" s="9"/>
-      <c r="L57" s="2">
+      <c r="L57" s="11">
         <v>6</v>
       </c>
-      <c r="M57" s="10"/>
-      <c r="N57" s="10"/>
+      <c r="M57" s="9"/>
+      <c r="N57" s="9"/>
       <c r="O57" s="9"/>
       <c r="P57" s="9"/>
-    </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q57" s="10"/>
+      <c r="R57" s="10"/>
+      <c r="S57" s="10"/>
+      <c r="T57" s="10"/>
+      <c r="U57" s="10"/>
+    </row>
+    <row r="58" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A58" s="9" t="s">
         <v>23</v>
       </c>
       <c r="B58" s="9"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="9"/>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
       <c r="H58" s="9"/>
-      <c r="I58" s="10"/>
+      <c r="I58" s="9"/>
       <c r="J58" s="9"/>
       <c r="K58" s="9"/>
-      <c r="L58" s="2">
+      <c r="L58" s="11">
         <v>6</v>
       </c>
-      <c r="M58" s="10"/>
-      <c r="N58" s="10"/>
+      <c r="M58" s="9"/>
+      <c r="N58" s="9"/>
       <c r="O58" s="9"/>
       <c r="P58" s="9"/>
+      <c r="Q58" s="10"/>
+      <c r="R58" s="10"/>
+      <c r="S58" s="10"/>
+      <c r="T58" s="10"/>
+      <c r="U58" s="10"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:P5 M7:P8 A7:K58">
-    <cfRule type="expression" dxfId="5" priority="5">
+  <conditionalFormatting sqref="A2:P58">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>COUNTA($A2:$P2)=COLUMNS($A2:$P2)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="4" priority="6">
+    <cfRule type="containsBlanks" dxfId="2" priority="2">
       <formula>LEN(TRIM(A2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M9:P58">
-    <cfRule type="expression" dxfId="3" priority="3">
-      <formula>COUNTA($A9:$P9)=COLUMNS($A9:$P9)</formula>
-    </cfRule>
-    <cfRule type="containsBlanks" dxfId="2" priority="4">
-      <formula>LEN(TRIM(M9))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6:P6">
-    <cfRule type="expression" dxfId="1" priority="1">
-      <formula>COUNTA($A6:$P6)=COLUMNS($A6:$P6)</formula>
-    </cfRule>
-    <cfRule type="containsBlanks" dxfId="0" priority="2">
-      <formula>LEN(TRIM(A6))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">

</xml_diff>

<commit_message>
Add doc for last group 2 rally
</commit_message>
<xml_diff>
--- a/Rallies.xlsx
+++ b/Rallies.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="92">
   <si>
     <t>Year</t>
   </si>
@@ -265,17 +265,38 @@
     <t>1, 8, 10, 5, 7</t>
   </si>
   <si>
-    <t>After dominating in the french rallies, &lt;b&gt;Jean-Claude Andruet&lt;/b&gt; wildly swong his &lt;b&gt;Alpine A110&lt;/b&gt; with &lt;b&gt;Michèle Veron&lt;/b&gt; as copilot in this rally spanning between Germany, Austria and Hungary. The battle with Fords and Porsches was fierce but they won the French and European rally championships titles.</t>
-  </si>
-  <si>
     <t>Rain, Morning, Rain, Sunset, Fog</t>
+  </si>
+  <si>
+    <t>East Germany</t>
+  </si>
+  <si>
+    <t>Pneumant Rallye</t>
+  </si>
+  <si>
+    <t>Sobiesław Zasada</t>
+  </si>
+  <si>
+    <t>17-20 March</t>
+  </si>
+  <si>
+    <t>After dominating in the french rallies, &lt;b&gt;Jean-Claude Andruet&lt;/b&gt; wildly swung his &lt;b&gt;Alpine A110&lt;/b&gt; with &lt;b&gt;Michèle Veron&lt;/b&gt; as copilot in this rally spanning between Germany, Austria and Hungary. The battle with Fords and Porsches was fierce but they won the French and European rally championships titles.</t>
+  </si>
+  <si>
+    <t>Out with the Porsche, in with a &lt;b&gt;BMW 2002 Ti&lt;/b&gt; that &lt;b&gt;Sobiesław Zasada&lt;/b&gt; hurls through the fog and rain of &lt;bWEast Germany&lt;/b&gt;, as if it was a javelin from his youth. Pairing up with copilot &lt;b&gt;Adam Wędrychowski&lt;/b&gt;, he ended up winning his third european champion in &lt;b&gt;1971&lt;/b&gt;, winning both the &lt;b&gt;East Germany&lt;/b&gt; and &lt;b&gt;Polish&lt;/b&gt; rally.</t>
+  </si>
+  <si>
+    <t>Fog,     Rain,   Rain, Afternoon, Fog, Sunset</t>
+  </si>
+  <si>
+    <t>7, 0, 9, 1, 8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -293,6 +314,14 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -336,10 +365,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -374,81 +404,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -765,15 +729,16 @@
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="7" style="1" customWidth="1"/>
-    <col min="3" max="4" width="9" style="3" customWidth="1"/>
+    <col min="3" max="3" width="9" style="3" customWidth="1"/>
+    <col min="4" max="4" width="9.54296875" style="3" customWidth="1"/>
     <col min="5" max="5" width="15.81640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.81640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="19" style="1" customWidth="1"/>
     <col min="8" max="8" width="12.1796875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="14.54296875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.26953125" style="1" customWidth="1"/>
     <col min="10" max="10" width="7.1796875" style="1" customWidth="1"/>
     <col min="11" max="11" width="12.26953125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="10.81640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.90625" style="1" customWidth="1"/>
     <col min="13" max="13" width="9.81640625" style="1" customWidth="1"/>
     <col min="14" max="14" width="62" style="1" customWidth="1"/>
     <col min="15" max="16" width="8.453125" style="1" customWidth="1"/>
@@ -1020,7 +985,7 @@
         <v>5</v>
       </c>
       <c r="K4" s="9">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L4" s="9" t="s">
         <v>67</v>
@@ -1055,7 +1020,7 @@
       <c r="X4" s="3"/>
       <c r="Y4" s="3"/>
     </row>
-    <row r="5" spans="1:25" ht="91" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:25" ht="81.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>12</v>
       </c>
@@ -1189,7 +1154,7 @@
       <c r="X6" s="3"/>
       <c r="Y6" s="3"/>
     </row>
-    <row r="7" spans="1:25" ht="84" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:25" ht="80" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>12</v>
       </c>
@@ -1227,10 +1192,10 @@
         <v>82</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N7" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="O7" s="9" t="s">
         <v>60</v>
@@ -1254,27 +1219,55 @@
       <c r="X7" s="3"/>
       <c r="Y7" s="3"/>
     </row>
-    <row r="8" spans="1:25" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:25" ht="91" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="11">
-        <v>6</v>
-      </c>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
+      <c r="B8" s="9">
+        <v>1971</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="H8" s="9">
+        <v>1971</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J8" s="9">
+        <v>2</v>
+      </c>
+      <c r="K8" s="9">
+        <v>0</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="M8" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="N8" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="O8" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="P8" s="9" t="s">
+        <v>60</v>
+      </c>
       <c r="Q8" s="10"/>
       <c r="R8" s="7" t="s">
         <v>18</v>
@@ -2685,10 +2678,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:P58">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>COUNTA($A2:$P2)=COLUMNS($A2:$P2)</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="2" priority="2">
+    <cfRule type="containsBlanks" dxfId="0" priority="2">
       <formula>LEN(TRIM(A2))=0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>